<commit_message>
feat(panel): decisiones delegadas para los 17 expedientes sin consenso
- 15 clases del contraste de 2.°–8.°, casi todas de umbral, resueltas con la
  regla «solo se afirma lo que coincide» y una cita literal de la fila de la
  V2: 10 alineadas, 3 posteriores (mareas, elasticidad, industria química) y
  2 fuera del contraste (especies clave, glaciaciones). El contraste de
  2.°–8.° ya no tiene conceptos inciertos.
- G07-CIE-U6-6.12 vuelve a Biología (alternativa de los dos expertos).
- Hallazgo del ciclo de las estrellas: se matiza con el texto del experto.
- Nueva solidez «delegada» (sin consenso del panel, decidido por el
  responsable con evidencia, pendiente de confirmar) en el informe, el CSV
  (190 decisiones) y los snapshots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_biologia.xlsx
+++ b/internacional/2_8/Contraste_biologia.xlsx
@@ -5820,7 +5820,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Nutrición autótrofa y heterótrofa</t>
+          <t>Niveles de organización ecológica</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5829,34 +5829,31 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>2.5</v>
       </c>
       <c r="G77" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H77" t="n">
-        <v>2</v>
-      </c>
-      <c r="I77" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J77" t="n">
         <v>2.5</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L77" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M77" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="O77" t="n">
         <v>1</v>
@@ -5867,9 +5864,6 @@
       <c r="Q77" t="n">
         <v>1</v>
       </c>
-      <c r="R77" t="n">
-        <v>1</v>
-      </c>
       <c r="S77" t="n">
         <v>1</v>
       </c>
@@ -5883,7 +5877,7 @@
         <v>1</v>
       </c>
       <c r="AF77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG77" t="inlineStr">
         <is>
@@ -5899,7 +5893,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Órganos de los sentidos</t>
+          <t>Nutrición autótrofa y heterótrofa</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -5908,13 +5902,13 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
@@ -5923,13 +5917,19 @@
         <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J78" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="K78" t="n">
+        <v>2</v>
+      </c>
+      <c r="L78" t="n">
+        <v>5</v>
       </c>
       <c r="M78" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="O78" t="n">
         <v>1</v>
@@ -5946,15 +5946,21 @@
       <c r="S78" t="n">
         <v>1</v>
       </c>
+      <c r="T78" t="n">
+        <v>1</v>
+      </c>
+      <c r="U78" t="n">
+        <v>1</v>
+      </c>
       <c r="V78" t="n">
         <v>1</v>
       </c>
       <c r="AF78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH78" t="inlineStr">
@@ -5966,7 +5972,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Partes de la planta y sus funciones</t>
+          <t>Órganos de los sentidos</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5975,16 +5981,13 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G79" t="n">
         <v>2</v>
@@ -5993,23 +5996,14 @@
         <v>2</v>
       </c>
       <c r="I79" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J79" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K79" t="n">
-        <v>2</v>
-      </c>
-      <c r="L79" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M79" t="n">
         <v>2.5</v>
       </c>
-      <c r="N79" t="n">
-        <v>1</v>
-      </c>
       <c r="O79" t="n">
         <v>1</v>
       </c>
@@ -6025,17 +6019,11 @@
       <c r="S79" t="n">
         <v>1</v>
       </c>
-      <c r="T79" t="n">
-        <v>1</v>
-      </c>
-      <c r="U79" t="n">
-        <v>1</v>
-      </c>
       <c r="V79" t="n">
         <v>1</v>
       </c>
       <c r="AF79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG79" t="inlineStr">
         <is>
@@ -6051,7 +6039,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Productores, consumidores y descomponedores</t>
+          <t>Partes de la planta y sus funciones</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -6060,13 +6048,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
         <v>2.5</v>
@@ -6075,10 +6063,10 @@
         <v>2</v>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I80" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J80" t="n">
         <v>2.5</v>
@@ -6087,10 +6075,10 @@
         <v>2</v>
       </c>
       <c r="L80" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M80" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="N80" t="n">
         <v>1</v>
@@ -6120,7 +6108,7 @@
         <v>1</v>
       </c>
       <c r="AF80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG80" t="inlineStr">
         <is>
@@ -6136,7 +6124,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Reproducción sexual de las plantas con flor</t>
+          <t>Plantas y animales útiles al ser humano</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -6145,37 +6133,28 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>6</v>
-      </c>
-      <c r="E81" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G81" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H81" t="n">
         <v>2</v>
       </c>
-      <c r="I81" t="n">
-        <v>4</v>
+      <c r="J81" t="n">
+        <v>2.5</v>
       </c>
       <c r="K81" t="n">
         <v>2</v>
       </c>
-      <c r="L81" t="n">
-        <v>5</v>
-      </c>
       <c r="M81" t="n">
-        <v>7</v>
-      </c>
-      <c r="N81" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="O81" t="n">
         <v>1</v>
@@ -6186,24 +6165,21 @@
       <c r="Q81" t="n">
         <v>1</v>
       </c>
-      <c r="R81" t="n">
+      <c r="S81" t="n">
         <v>1</v>
       </c>
       <c r="T81" t="n">
         <v>1</v>
       </c>
-      <c r="U81" t="n">
-        <v>1</v>
-      </c>
       <c r="V81" t="n">
         <v>1</v>
       </c>
       <c r="AF81" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AG81" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH81" t="inlineStr">
@@ -6215,7 +6191,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Reproducción humana y pubertad</t>
+          <t>Productores, consumidores y descomponedores</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6224,62 +6200,71 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E82" t="n">
+        <v>3</v>
+      </c>
+      <c r="F82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G82" t="n">
+        <v>2</v>
+      </c>
+      <c r="H82" t="n">
+        <v>3</v>
+      </c>
+      <c r="I82" t="n">
         <v>8</v>
       </c>
-      <c r="F82" t="n">
-        <v>8</v>
-      </c>
-      <c r="G82" t="n">
+      <c r="J82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K82" t="n">
+        <v>2</v>
+      </c>
+      <c r="L82" t="n">
+        <v>6</v>
+      </c>
+      <c r="M82" t="n">
+        <v>7</v>
+      </c>
+      <c r="N82" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" t="n">
+        <v>1</v>
+      </c>
+      <c r="P82" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>1</v>
+      </c>
+      <c r="R82" t="n">
+        <v>1</v>
+      </c>
+      <c r="S82" t="n">
+        <v>1</v>
+      </c>
+      <c r="T82" t="n">
+        <v>1</v>
+      </c>
+      <c r="U82" t="n">
+        <v>1</v>
+      </c>
+      <c r="V82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF82" t="n">
         <v>3</v>
       </c>
-      <c r="H82" t="n">
-        <v>4</v>
-      </c>
-      <c r="I82" t="n">
-        <v>4</v>
-      </c>
-      <c r="L82" t="n">
-        <v>5</v>
-      </c>
-      <c r="M82" t="n">
-        <v>7</v>
-      </c>
-      <c r="N82" t="n">
-        <v>1</v>
-      </c>
-      <c r="O82" t="n">
-        <v>1</v>
-      </c>
-      <c r="P82" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q82" t="n">
-        <v>1</v>
-      </c>
-      <c r="R82" t="n">
-        <v>1</v>
-      </c>
-      <c r="U82" t="n">
-        <v>1</v>
-      </c>
-      <c r="V82" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z82" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF82" t="n">
-        <v>4</v>
-      </c>
       <c r="AG82" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH82" t="inlineStr">
@@ -6291,7 +6276,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Reproducción sexual y asexual</t>
+          <t>Reproducción sexual de las plantas con flor</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6312,19 +6297,22 @@
         <v>8</v>
       </c>
       <c r="G83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I83" t="n">
         <v>4</v>
       </c>
+      <c r="K83" t="n">
+        <v>2</v>
+      </c>
       <c r="L83" t="n">
         <v>5</v>
       </c>
       <c r="M83" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="N83" t="n">
         <v>1</v>
@@ -6341,13 +6329,13 @@
       <c r="R83" t="n">
         <v>1</v>
       </c>
+      <c r="T83" t="n">
+        <v>1</v>
+      </c>
       <c r="U83" t="n">
         <v>1</v>
       </c>
       <c r="V83" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z83" t="n">
         <v>1</v>
       </c>
       <c r="AF83" t="n">
@@ -6367,7 +6355,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Requerimientos de materia y energía de la célula</t>
+          <t>Reproducción humana y pubertad</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6376,22 +6364,25 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="E84" t="n">
+        <v>8</v>
+      </c>
+      <c r="F84" t="n">
+        <v>8</v>
       </c>
       <c r="G84" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H84" t="n">
-        <v>7</v>
-      </c>
-      <c r="J84" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K84" t="n">
-        <v>7</v>
+        <v>4</v>
+      </c>
+      <c r="I84" t="n">
+        <v>4</v>
       </c>
       <c r="L84" t="n">
         <v>5</v>
@@ -6399,16 +6390,19 @@
       <c r="M84" t="n">
         <v>7</v>
       </c>
+      <c r="N84" t="n">
+        <v>1</v>
+      </c>
+      <c r="O84" t="n">
+        <v>1</v>
+      </c>
       <c r="P84" t="n">
         <v>1</v>
       </c>
       <c r="Q84" t="n">
         <v>1</v>
       </c>
-      <c r="S84" t="n">
-        <v>1</v>
-      </c>
-      <c r="T84" t="n">
+      <c r="R84" t="n">
         <v>1</v>
       </c>
       <c r="U84" t="n">
@@ -6421,11 +6415,11 @@
         <v>1</v>
       </c>
       <c r="AF84" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH84" t="inlineStr">
@@ -6437,7 +6431,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Antibióticos y resistencia bacteriana</t>
+          <t>Reproducción sexual y asexual</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6446,19 +6440,37 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D85" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="E85" t="n">
+        <v>8</v>
+      </c>
+      <c r="F85" t="n">
+        <v>8</v>
       </c>
       <c r="G85" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="H85" t="n">
+        <v>3</v>
+      </c>
+      <c r="I85" t="n">
         <v>4</v>
       </c>
       <c r="L85" t="n">
-        <v>7.5</v>
+        <v>5</v>
+      </c>
+      <c r="M85" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N85" t="n">
+        <v>1</v>
+      </c>
+      <c r="O85" t="n">
+        <v>1</v>
       </c>
       <c r="P85" t="n">
         <v>1</v>
@@ -6466,14 +6478,20 @@
       <c r="Q85" t="n">
         <v>1</v>
       </c>
+      <c r="R85" t="n">
+        <v>1</v>
+      </c>
       <c r="U85" t="n">
         <v>1</v>
       </c>
+      <c r="V85" t="n">
+        <v>1</v>
+      </c>
       <c r="Z85" t="n">
         <v>1</v>
       </c>
       <c r="AF85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
@@ -6489,7 +6507,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Respiración celular</t>
+          <t>Requerimientos de materia y energía de la célula</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -6503,48 +6521,30 @@
       <c r="D86" t="n">
         <v>6</v>
       </c>
-      <c r="E86" t="n">
-        <v>8</v>
-      </c>
-      <c r="F86" t="n">
-        <v>5</v>
-      </c>
       <c r="G86" t="n">
         <v>6</v>
       </c>
       <c r="H86" t="n">
         <v>7</v>
       </c>
-      <c r="I86" t="n">
-        <v>7</v>
-      </c>
       <c r="J86" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="K86" t="n">
         <v>7</v>
       </c>
       <c r="L86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M86" t="n">
         <v>7</v>
       </c>
-      <c r="N86" t="n">
-        <v>1</v>
-      </c>
-      <c r="O86" t="n">
-        <v>1</v>
-      </c>
       <c r="P86" t="n">
         <v>1</v>
       </c>
       <c r="Q86" t="n">
         <v>1</v>
       </c>
-      <c r="R86" t="n">
-        <v>1</v>
-      </c>
       <c r="S86" t="n">
         <v>1</v>
       </c>
@@ -6555,6 +6555,9 @@
         <v>1</v>
       </c>
       <c r="V86" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z86" t="n">
         <v>1</v>
       </c>
       <c r="AF86" t="n">
@@ -6562,7 +6565,7 @@
       </c>
       <c r="AG86" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH86" t="inlineStr">
@@ -6574,7 +6577,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Respuesta de los seres vivos a estímulos</t>
+          <t>Antibióticos y resistencia bacteriana</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6583,43 +6586,19 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
-      </c>
-      <c r="E87" t="n">
-        <v>8</v>
-      </c>
-      <c r="F87" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G87" t="n">
         <v>8.5</v>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
-      </c>
-      <c r="I87" t="n">
-        <v>3</v>
-      </c>
-      <c r="J87" t="n">
-        <v>7</v>
-      </c>
-      <c r="K87" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L87" t="n">
-        <v>3</v>
-      </c>
-      <c r="M87" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N87" t="n">
-        <v>1</v>
-      </c>
-      <c r="O87" t="n">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="P87" t="n">
         <v>1</v>
@@ -6627,27 +6606,18 @@
       <c r="Q87" t="n">
         <v>1</v>
       </c>
-      <c r="R87" t="n">
-        <v>1</v>
-      </c>
-      <c r="S87" t="n">
-        <v>1</v>
-      </c>
-      <c r="T87" t="n">
-        <v>1</v>
-      </c>
       <c r="U87" t="n">
         <v>1</v>
       </c>
-      <c r="V87" t="n">
+      <c r="Z87" t="n">
         <v>1</v>
       </c>
       <c r="AF87" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH87" t="inlineStr">
@@ -6659,7 +6629,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Modelo estímulo-respuesta y retroalimentación negativa</t>
+          <t>Respiración celular</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -6668,16 +6638,19 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D88" t="n">
+        <v>6</v>
       </c>
       <c r="E88" t="n">
         <v>8</v>
       </c>
       <c r="F88" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H88" t="n">
         <v>7</v>
@@ -6688,8 +6661,14 @@
       <c r="J88" t="n">
         <v>7</v>
       </c>
+      <c r="K88" t="n">
+        <v>7</v>
+      </c>
+      <c r="L88" t="n">
+        <v>6</v>
+      </c>
       <c r="M88" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="N88" t="n">
         <v>1</v>
@@ -6709,11 +6688,17 @@
       <c r="S88" t="n">
         <v>1</v>
       </c>
+      <c r="T88" t="n">
+        <v>1</v>
+      </c>
+      <c r="U88" t="n">
+        <v>1</v>
+      </c>
       <c r="V88" t="n">
         <v>1</v>
       </c>
       <c r="AF88" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AG88" t="inlineStr">
         <is>
@@ -6729,7 +6714,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Selección natural</t>
+          <t>Respuesta de los seres vivos a estímulos</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6738,22 +6723,40 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D89" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="E89" t="n">
+        <v>8</v>
       </c>
       <c r="F89" t="n">
         <v>8</v>
       </c>
       <c r="G89" t="n">
-        <v>4</v>
+        <v>8.5</v>
+      </c>
+      <c r="H89" t="n">
+        <v>2</v>
+      </c>
+      <c r="I89" t="n">
+        <v>3</v>
+      </c>
+      <c r="J89" t="n">
+        <v>7</v>
       </c>
       <c r="K89" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L89" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="M89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N89" t="n">
+        <v>1</v>
       </c>
       <c r="O89" t="n">
         <v>1</v>
@@ -6761,21 +6764,30 @@
       <c r="P89" t="n">
         <v>1</v>
       </c>
+      <c r="Q89" t="n">
+        <v>1</v>
+      </c>
+      <c r="R89" t="n">
+        <v>1</v>
+      </c>
+      <c r="S89" t="n">
+        <v>1</v>
+      </c>
       <c r="T89" t="n">
         <v>1</v>
       </c>
       <c r="U89" t="n">
         <v>1</v>
       </c>
-      <c r="Z89" t="n">
+      <c r="V89" t="n">
         <v>1</v>
       </c>
       <c r="AF89" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG89" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH89" t="inlineStr">
@@ -6787,7 +6799,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Seres vivos y no vivos</t>
+          <t>Modelo estímulo-respuesta y retroalimentación negativa</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6796,28 +6808,28 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2</v>
-      </c>
-      <c r="D90" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F90" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G90" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H90" t="n">
-        <v>2</v>
-      </c>
-      <c r="L90" t="n">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="I90" t="n">
+        <v>7</v>
+      </c>
+      <c r="J90" t="n">
+        <v>7</v>
       </c>
       <c r="M90" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="N90" t="n">
         <v>1</v>
@@ -6831,14 +6843,17 @@
       <c r="Q90" t="n">
         <v>1</v>
       </c>
-      <c r="U90" t="n">
+      <c r="R90" t="n">
+        <v>1</v>
+      </c>
+      <c r="S90" t="n">
         <v>1</v>
       </c>
       <c r="V90" t="n">
         <v>1</v>
       </c>
       <c r="AF90" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AG90" t="inlineStr">
         <is>
@@ -6854,7 +6869,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Sistema circulatorio</t>
+          <t>Selección natural</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6863,10 +6878,10 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D91" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>8</v>
@@ -6874,23 +6889,11 @@
       <c r="G91" t="n">
         <v>4</v>
       </c>
-      <c r="H91" t="n">
-        <v>2</v>
-      </c>
-      <c r="I91" t="n">
+      <c r="K91" t="n">
         <v>5</v>
       </c>
-      <c r="J91" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K91" t="n">
-        <v>4</v>
-      </c>
       <c r="L91" t="n">
-        <v>4</v>
-      </c>
-      <c r="M91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O91" t="n">
         <v>1</v>
@@ -6898,29 +6901,17 @@
       <c r="P91" t="n">
         <v>1</v>
       </c>
-      <c r="Q91" t="n">
-        <v>1</v>
-      </c>
-      <c r="R91" t="n">
-        <v>1</v>
-      </c>
-      <c r="S91" t="n">
-        <v>1</v>
-      </c>
       <c r="T91" t="n">
         <v>1</v>
       </c>
       <c r="U91" t="n">
         <v>1</v>
       </c>
-      <c r="V91" t="n">
-        <v>1</v>
-      </c>
       <c r="Z91" t="n">
         <v>1</v>
       </c>
       <c r="AF91" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AG91" t="inlineStr">
         <is>
@@ -6936,7 +6927,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Sistema digestivo</t>
+          <t>Seres vivos y no vivos</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6945,34 +6936,31 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D92" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="E92" t="n">
+        <v>2</v>
       </c>
       <c r="F92" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G92" t="n">
         <v>2</v>
       </c>
       <c r="H92" t="n">
-        <v>4</v>
-      </c>
-      <c r="I92" t="n">
-        <v>5</v>
-      </c>
-      <c r="J92" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K92" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M92" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="N92" t="n">
+        <v>1</v>
       </c>
       <c r="O92" t="n">
         <v>1</v>
@@ -6983,26 +6971,14 @@
       <c r="Q92" t="n">
         <v>1</v>
       </c>
-      <c r="R92" t="n">
-        <v>1</v>
-      </c>
-      <c r="S92" t="n">
-        <v>1</v>
-      </c>
-      <c r="T92" t="n">
-        <v>1</v>
-      </c>
       <c r="U92" t="n">
         <v>1</v>
       </c>
       <c r="V92" t="n">
         <v>1</v>
       </c>
-      <c r="Z92" t="n">
-        <v>1</v>
-      </c>
       <c r="AF92" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG92" t="inlineStr">
         <is>
@@ -7018,7 +6994,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Sistema endocrino y hormonas</t>
+          <t>Sistema circulatorio</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -7027,38 +7003,53 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>9</v>
-      </c>
-      <c r="E93" t="n">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="D93" t="n">
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>8</v>
       </c>
       <c r="G93" t="n">
-        <v>8.5</v>
+        <v>4</v>
+      </c>
+      <c r="H93" t="n">
+        <v>2</v>
+      </c>
+      <c r="I93" t="n">
+        <v>5</v>
       </c>
       <c r="J93" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K93" t="n">
+        <v>4</v>
       </c>
       <c r="L93" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="M93" t="n">
         <v>7</v>
       </c>
-      <c r="N93" t="n">
-        <v>1</v>
-      </c>
       <c r="O93" t="n">
         <v>1</v>
       </c>
       <c r="P93" t="n">
         <v>1</v>
       </c>
+      <c r="Q93" t="n">
+        <v>1</v>
+      </c>
+      <c r="R93" t="n">
+        <v>1</v>
+      </c>
       <c r="S93" t="n">
         <v>1</v>
       </c>
+      <c r="T93" t="n">
+        <v>1</v>
+      </c>
       <c r="U93" t="n">
         <v>1</v>
       </c>
@@ -7069,7 +7060,7 @@
         <v>1</v>
       </c>
       <c r="AF93" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AG93" t="inlineStr">
         <is>
@@ -7085,7 +7076,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Sistema locomotor</t>
+          <t>Sistema digestivo</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7106,16 +7097,22 @@
         <v>2</v>
       </c>
       <c r="H94" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I94" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J94" t="n">
         <v>4.5</v>
       </c>
+      <c r="K94" t="n">
+        <v>4</v>
+      </c>
+      <c r="L94" t="n">
+        <v>4</v>
+      </c>
       <c r="M94" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="O94" t="n">
         <v>1</v>
@@ -7132,7 +7129,16 @@
       <c r="S94" t="n">
         <v>1</v>
       </c>
+      <c r="T94" t="n">
+        <v>1</v>
+      </c>
+      <c r="U94" t="n">
+        <v>1</v>
+      </c>
       <c r="V94" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z94" t="n">
         <v>1</v>
       </c>
       <c r="AF94" t="n">
@@ -7152,7 +7158,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Sistema respiratorio</t>
+          <t>Sistema endocrino y hormonas</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -7161,53 +7167,38 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
-      </c>
-      <c r="D95" t="n">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="E95" t="n">
+        <v>8</v>
       </c>
       <c r="F95" t="n">
         <v>8</v>
       </c>
       <c r="G95" t="n">
-        <v>6</v>
-      </c>
-      <c r="H95" t="n">
-        <v>2</v>
-      </c>
-      <c r="I95" t="n">
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="J95" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K95" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L95" t="n">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="M95" t="n">
         <v>7</v>
       </c>
+      <c r="N95" t="n">
+        <v>1</v>
+      </c>
       <c r="O95" t="n">
         <v>1</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
       </c>
-      <c r="Q95" t="n">
-        <v>1</v>
-      </c>
-      <c r="R95" t="n">
-        <v>1</v>
-      </c>
       <c r="S95" t="n">
         <v>1</v>
       </c>
-      <c r="T95" t="n">
-        <v>1</v>
-      </c>
       <c r="U95" t="n">
         <v>1</v>
       </c>
@@ -7218,11 +7209,11 @@
         <v>1</v>
       </c>
       <c r="AF95" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AG95" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH95" t="inlineStr">
@@ -7234,7 +7225,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Tejidos animales</t>
+          <t>Sistema locomotor</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -7248,20 +7239,23 @@
       <c r="D96" t="n">
         <v>4</v>
       </c>
-      <c r="E96" t="n">
-        <v>7</v>
-      </c>
       <c r="F96" t="n">
         <v>8</v>
       </c>
       <c r="G96" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H96" t="n">
-        <v>7</v>
-      </c>
-      <c r="N96" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I96" t="n">
+        <v>3</v>
+      </c>
+      <c r="J96" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M96" t="n">
+        <v>4.5</v>
       </c>
       <c r="O96" t="n">
         <v>1</v>
@@ -7272,7 +7266,13 @@
       <c r="Q96" t="n">
         <v>1</v>
       </c>
-      <c r="Z96" t="n">
+      <c r="R96" t="n">
+        <v>1</v>
+      </c>
+      <c r="S96" t="n">
+        <v>1</v>
+      </c>
+      <c r="V96" t="n">
         <v>1</v>
       </c>
       <c r="AF96" t="n">
@@ -7280,19 +7280,19 @@
       </c>
       <c r="AG96" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH96" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Tejidos vegetales</t>
+          <t>Sistema respiratorio</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -7301,35 +7301,35 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>8</v>
-      </c>
-      <c r="E97" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
         <v>8</v>
       </c>
       <c r="G97" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H97" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="I97" t="n">
+        <v>5</v>
       </c>
       <c r="J97" t="n">
         <v>4.5</v>
       </c>
+      <c r="K97" t="n">
+        <v>4</v>
+      </c>
       <c r="L97" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="M97" t="n">
         <v>7</v>
       </c>
-      <c r="N97" t="n">
-        <v>1</v>
-      </c>
       <c r="O97" t="n">
         <v>1</v>
       </c>
@@ -7339,21 +7339,30 @@
       <c r="Q97" t="n">
         <v>1</v>
       </c>
+      <c r="R97" t="n">
+        <v>1</v>
+      </c>
       <c r="S97" t="n">
         <v>1</v>
       </c>
+      <c r="T97" t="n">
+        <v>1</v>
+      </c>
       <c r="U97" t="n">
         <v>1</v>
       </c>
       <c r="V97" t="n">
         <v>1</v>
       </c>
+      <c r="Z97" t="n">
+        <v>1</v>
+      </c>
       <c r="AF97" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AG97" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH97" t="inlineStr">
@@ -7365,7 +7374,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Transporte en plantas: xilema y floema</t>
+          <t>Tejidos animales</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -7374,28 +7383,28 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D98" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="E98" t="n">
+        <v>7</v>
+      </c>
+      <c r="F98" t="n">
+        <v>8</v>
       </c>
       <c r="G98" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H98" t="n">
         <v>7</v>
       </c>
-      <c r="I98" t="n">
-        <v>5</v>
-      </c>
-      <c r="J98" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L98" t="n">
-        <v>5</v>
-      </c>
-      <c r="M98" t="n">
-        <v>7</v>
+      <c r="N98" t="n">
+        <v>1</v>
+      </c>
+      <c r="O98" t="n">
+        <v>1</v>
       </c>
       <c r="P98" t="n">
         <v>1</v>
@@ -7403,36 +7412,27 @@
       <c r="Q98" t="n">
         <v>1</v>
       </c>
-      <c r="R98" t="n">
-        <v>1</v>
-      </c>
-      <c r="S98" t="n">
-        <v>1</v>
-      </c>
-      <c r="U98" t="n">
-        <v>1</v>
-      </c>
-      <c r="V98" t="n">
+      <c r="Z98" t="n">
         <v>1</v>
       </c>
       <c r="AF98" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AG98" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH98" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Variación genética en la descendencia</t>
+          <t>Tejidos vegetales</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -7441,31 +7441,34 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D99" t="n">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="E99" t="n">
+        <v>7</v>
       </c>
       <c r="F99" t="n">
         <v>8</v>
       </c>
       <c r="G99" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="H99" t="n">
         <v>7</v>
       </c>
-      <c r="I99" t="n">
-        <v>8</v>
-      </c>
-      <c r="K99" t="n">
-        <v>5</v>
+      <c r="J99" t="n">
+        <v>4.5</v>
       </c>
       <c r="L99" t="n">
         <v>7.5</v>
       </c>
       <c r="M99" t="n">
-        <v>4.5</v>
+        <v>7</v>
+      </c>
+      <c r="N99" t="n">
+        <v>1</v>
       </c>
       <c r="O99" t="n">
         <v>1</v>
@@ -7476,10 +7479,7 @@
       <c r="Q99" t="n">
         <v>1</v>
       </c>
-      <c r="R99" t="n">
-        <v>1</v>
-      </c>
-      <c r="T99" t="n">
+      <c r="S99" t="n">
         <v>1</v>
       </c>
       <c r="U99" t="n">
@@ -7489,7 +7489,7 @@
         <v>1</v>
       </c>
       <c r="AF99" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG99" t="inlineStr">
         <is>
@@ -7505,71 +7505,104 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Especies clave</t>
+          <t>Transporte en plantas: xilema y floema</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D100" t="n">
-        <v>7</v>
-      </c>
-      <c r="K100" t="n">
-        <v>3</v>
-      </c>
-      <c r="T100" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="G100" t="n">
+        <v>2</v>
+      </c>
+      <c r="H100" t="n">
+        <v>7</v>
+      </c>
+      <c r="I100" t="n">
+        <v>5</v>
+      </c>
+      <c r="J100" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L100" t="n">
+        <v>5</v>
+      </c>
+      <c r="M100" t="n">
+        <v>7</v>
+      </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>1</v>
+      </c>
+      <c r="R100" t="n">
+        <v>1</v>
+      </c>
+      <c r="S100" t="n">
+        <v>1</v>
+      </c>
+      <c r="U100" t="n">
+        <v>1</v>
+      </c>
+      <c r="V100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>8</v>
       </c>
       <c r="AG100" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH100" t="inlineStr">
         <is>
-          <t>no_aplica</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Niveles de organización ecológica</t>
+          <t>Variación genética en la descendencia</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C101" t="n">
+        <v>6</v>
+      </c>
+      <c r="D101" t="n">
+        <v>6</v>
+      </c>
+      <c r="F101" t="n">
+        <v>8</v>
+      </c>
+      <c r="G101" t="n">
         <v>4</v>
       </c>
-      <c r="D101" t="n">
-        <v>4</v>
-      </c>
-      <c r="F101" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G101" t="n">
-        <v>8.5</v>
-      </c>
       <c r="H101" t="n">
-        <v>3</v>
-      </c>
-      <c r="J101" t="n">
-        <v>2.5</v>
+        <v>7</v>
+      </c>
+      <c r="I101" t="n">
+        <v>8</v>
       </c>
       <c r="K101" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L101" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="M101" t="n">
         <v>4.5</v>
@@ -7583,7 +7616,7 @@
       <c r="Q101" t="n">
         <v>1</v>
       </c>
-      <c r="S101" t="n">
+      <c r="R101" t="n">
         <v>1</v>
       </c>
       <c r="T101" t="n">
@@ -7596,11 +7629,11 @@
         <v>1</v>
       </c>
       <c r="AF101" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AG101" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH101" t="inlineStr">
@@ -7612,67 +7645,34 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Plantas y animales útiles al ser humano</t>
+          <t>Especies clave</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>no_aplica</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D102" t="n">
-        <v>2</v>
-      </c>
-      <c r="F102" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G102" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H102" t="n">
-        <v>2</v>
-      </c>
-      <c r="J102" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="K102" t="n">
-        <v>2</v>
-      </c>
-      <c r="M102" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="O102" t="n">
-        <v>1</v>
-      </c>
-      <c r="P102" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q102" t="n">
-        <v>1</v>
-      </c>
-      <c r="S102" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T102" t="n">
         <v>1</v>
       </c>
-      <c r="V102" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF102" t="n">
-        <v>2</v>
-      </c>
       <c r="AG102" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH102" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>no_aplica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(internacional): Ontario Grades 1–2 en el contraste de 2.°–8.°
- Extraídos con Vertex (gasto aprobado: 29 llamadas de extracción y 19 de
  etiquetado) 85 objetivos de ON Grades 1–2, llevados a SV 2 como HK P1–P3.
- Cambian 4 clases: el ciclo del agua pasa a alineado; grupos de vertebrados,
  energía cinética y tono y volumen del sonido quedaron inciertos y se
  resolvieron como alineados por decisión delegada con su cita literal.
- Bug: extraer reescribía los objetivos desde la caché y borraba las
  correcciones de metadatos (Extension Part de HK); ahora vuelve a correr
  corregir-metadatos al terminar.
- El CLI aclara que el conteo previo de llamadas es una cota inferior y
  sugiere pedir aprobación con +25 %.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_biologia.xlsx
+++ b/internacional/2_8/Contraste_biologia.xlsx
@@ -922,7 +922,7 @@
         <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
         <v>6</v>
@@ -1848,7 +1848,7 @@
         <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
         <v>7.5</v>
@@ -2270,6 +2270,9 @@
       <c r="J26" t="n">
         <v>2.5</v>
       </c>
+      <c r="K26" t="n">
+        <v>2</v>
+      </c>
       <c r="L26" t="n">
         <v>6</v>
       </c>
@@ -2294,6 +2297,9 @@
       <c r="S26" t="n">
         <v>1</v>
       </c>
+      <c r="T26" t="n">
+        <v>1</v>
+      </c>
       <c r="U26" t="n">
         <v>1</v>
       </c>
@@ -2988,6 +2994,9 @@
       <c r="J36" t="n">
         <v>2.5</v>
       </c>
+      <c r="K36" t="n">
+        <v>2</v>
+      </c>
       <c r="L36" t="n">
         <v>3</v>
       </c>
@@ -3012,6 +3021,9 @@
       <c r="S36" t="n">
         <v>1</v>
       </c>
+      <c r="T36" t="n">
+        <v>1</v>
+      </c>
       <c r="U36" t="n">
         <v>1</v>
       </c>
@@ -3062,7 +3074,7 @@
         <v>4.5</v>
       </c>
       <c r="K37" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
         <v>5</v>
@@ -3138,7 +3150,7 @@
         <v>4.5</v>
       </c>
       <c r="K38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L38" t="n">
         <v>7.5</v>
@@ -3275,7 +3287,7 @@
         <v>2.5</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L40" t="n">
         <v>3</v>
@@ -4186,7 +4198,7 @@
         <v>2.5</v>
       </c>
       <c r="K54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
         <v>4</v>
@@ -4977,7 +4989,7 @@
         <v>4</v>
       </c>
       <c r="K65" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M65" t="n">
         <v>2.5</v>
@@ -5005,7 +5017,7 @@
       </c>
       <c r="AG65" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH65" t="inlineStr">
@@ -5533,6 +5545,9 @@
       <c r="I73" t="n">
         <v>2</v>
       </c>
+      <c r="K73" t="n">
+        <v>2</v>
+      </c>
       <c r="O73" t="n">
         <v>1</v>
       </c>
@@ -5543,6 +5558,9 @@
         <v>1</v>
       </c>
       <c r="R73" t="n">
+        <v>1</v>
+      </c>
+      <c r="T73" t="n">
         <v>1</v>
       </c>
       <c r="AF73" t="n">
@@ -6001,6 +6019,9 @@
       <c r="J79" t="n">
         <v>7</v>
       </c>
+      <c r="K79" t="n">
+        <v>2</v>
+      </c>
       <c r="M79" t="n">
         <v>2.5</v>
       </c>
@@ -6019,6 +6040,9 @@
       <c r="S79" t="n">
         <v>1</v>
       </c>
+      <c r="T79" t="n">
+        <v>1</v>
+      </c>
       <c r="V79" t="n">
         <v>1</v>
       </c>
@@ -6890,7 +6914,7 @@
         <v>4</v>
       </c>
       <c r="K91" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L91" t="n">
         <v>6</v>
@@ -6953,6 +6977,9 @@
       <c r="H92" t="n">
         <v>2</v>
       </c>
+      <c r="K92" t="n">
+        <v>2</v>
+      </c>
       <c r="L92" t="n">
         <v>3</v>
       </c>
@@ -6971,6 +6998,9 @@
       <c r="Q92" t="n">
         <v>1</v>
       </c>
+      <c r="T92" t="n">
+        <v>1</v>
+      </c>
       <c r="U92" t="n">
         <v>1</v>
       </c>
@@ -7254,6 +7284,9 @@
       <c r="J96" t="n">
         <v>4.5</v>
       </c>
+      <c r="K96" t="n">
+        <v>2</v>
+      </c>
       <c r="M96" t="n">
         <v>4.5</v>
       </c>
@@ -7272,6 +7305,9 @@
       <c r="S96" t="n">
         <v>1</v>
       </c>
+      <c r="T96" t="n">
+        <v>1</v>
+      </c>
       <c r="V96" t="n">
         <v>1</v>
       </c>
@@ -7697,7 +7733,7 @@
         <v>3</v>
       </c>
       <c r="K103" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O103" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
fix(internacional): ajustes de la búsqueda de texto del contraste
contraste.AJUSTES_BUSQUEDA quita frases que en la malla encuentran otra cosa
(«reacción en cadena» → la PCR; «ángulo crítico» y «punto crítico» → el
pensamiento crítico; «diagramas de fases» → las fases de la Luna; «ciclos
sedimentarios» → el ciclo de las rocas; «constante de tiempo»,
«cuantización de la energía», «interacciones fundamentales») y agrega
«virus infecciosos». Solo afecta la búsqueda del contraste.
- 9.°–11.°: 7 clases automáticas pasan a coincidir con las del panel.
- 2.°–8.°: 5 conceptos que solo entraban por coincidencias falsas salen del
  contraste; virus queda «posterior» por decisión delegada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_biologia.xlsx
+++ b/internacional/2_8/Contraste_biologia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH152"/>
+  <dimension ref="A1:AH151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -7841,7 +7841,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Ciclos del fósforo y del azufre</t>
+          <t>Propagación de enfermedades y control de brotes</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -7850,17 +7850,41 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
-      </c>
-      <c r="D106" t="n">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="G106" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H106" t="n">
+        <v>3</v>
+      </c>
+      <c r="J106" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L106" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P106" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>1</v>
+      </c>
+      <c r="S106" t="n">
+        <v>1</v>
+      </c>
+      <c r="U106" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z106" t="n">
+        <v>1</v>
       </c>
       <c r="AF106" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG106" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH106" t="inlineStr">
@@ -7872,7 +7896,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Propagación de enfermedades y control de brotes</t>
+          <t>Especiación y macroevolución</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -7881,37 +7905,22 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F107" t="n">
+        <v>8</v>
       </c>
       <c r="G107" t="n">
         <v>8.5</v>
       </c>
-      <c r="H107" t="n">
-        <v>3</v>
-      </c>
-      <c r="J107" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L107" t="n">
-        <v>7.5</v>
+      <c r="O107" t="n">
+        <v>1</v>
       </c>
       <c r="P107" t="n">
         <v>1</v>
       </c>
-      <c r="Q107" t="n">
-        <v>1</v>
-      </c>
-      <c r="S107" t="n">
-        <v>1</v>
-      </c>
-      <c r="U107" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z107" t="n">
-        <v>1</v>
-      </c>
       <c r="AF107" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG107" t="inlineStr">
         <is>
@@ -7927,7 +7936,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Especiación y macroevolución</t>
+          <t>Eutrofización</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -7936,26 +7945,17 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
-      </c>
-      <c r="F108" t="n">
-        <v>8</v>
-      </c>
-      <c r="G108" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="O108" t="n">
-        <v>1</v>
-      </c>
-      <c r="P108" t="n">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="D108" t="n">
+        <v>7</v>
       </c>
       <c r="AF108" t="n">
         <v>10</v>
       </c>
       <c r="AG108" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH108" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Eutrofización</t>
+          <t>Evidencias de la evolución</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -7976,17 +7976,38 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>7</v>
-      </c>
-      <c r="D109" t="n">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="F109" t="n">
+        <v>8</v>
+      </c>
+      <c r="G109" t="n">
+        <v>4</v>
+      </c>
+      <c r="I109" t="n">
+        <v>8</v>
+      </c>
+      <c r="M109" t="n">
+        <v>7</v>
+      </c>
+      <c r="O109" t="n">
+        <v>1</v>
+      </c>
+      <c r="P109" t="n">
+        <v>1</v>
+      </c>
+      <c r="R109" t="n">
+        <v>1</v>
+      </c>
+      <c r="V109" t="n">
+        <v>1</v>
       </c>
       <c r="AF109" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH109" t="inlineStr">
@@ -7998,7 +8019,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Evidencias de la evolución</t>
+          <t>Fases de la fotosíntesis y ciclo de Calvin</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -8007,38 +8028,23 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D110" t="n">
+        <v>6</v>
       </c>
       <c r="F110" t="n">
         <v>8</v>
       </c>
-      <c r="G110" t="n">
-        <v>4</v>
-      </c>
-      <c r="I110" t="n">
-        <v>8</v>
-      </c>
-      <c r="M110" t="n">
-        <v>7</v>
-      </c>
       <c r="O110" t="n">
         <v>1</v>
       </c>
-      <c r="P110" t="n">
-        <v>1</v>
-      </c>
-      <c r="R110" t="n">
-        <v>1</v>
-      </c>
-      <c r="V110" t="n">
-        <v>1</v>
-      </c>
       <c r="AF110" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG110" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH110" t="inlineStr">
@@ -8050,7 +8056,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Fases de la fotosíntesis y ciclo de Calvin</t>
+          <t>Secuenciación del ADN y perfiles genéticos</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -8059,15 +8065,18 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>6</v>
-      </c>
-      <c r="D111" t="n">
-        <v>6</v>
-      </c>
-      <c r="F111" t="n">
-        <v>8</v>
-      </c>
-      <c r="O111" t="n">
+        <v>9</v>
+      </c>
+      <c r="G111" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H111" t="n">
+        <v>7</v>
+      </c>
+      <c r="P111" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q111" t="n">
         <v>1</v>
       </c>
       <c r="AF111" t="n">
@@ -8075,7 +8084,7 @@
       </c>
       <c r="AG111" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH111" t="inlineStr">
@@ -8087,7 +8096,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Secuenciación del ADN y perfiles genéticos</t>
+          <t>Impulso nervioso y sinapsis</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -8096,18 +8105,18 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>9</v>
-      </c>
-      <c r="G112" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H112" t="n">
-        <v>7</v>
-      </c>
-      <c r="P112" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q112" t="n">
+        <v>10</v>
+      </c>
+      <c r="F112" t="n">
+        <v>8</v>
+      </c>
+      <c r="J112" t="n">
+        <v>7</v>
+      </c>
+      <c r="O112" t="n">
+        <v>1</v>
+      </c>
+      <c r="S112" t="n">
         <v>1</v>
       </c>
       <c r="AF112" t="n">
@@ -8127,7 +8136,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Impulso nervioso y sinapsis</t>
+          <t>Ingeniería genética y ADN recombinante</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8136,22 +8145,37 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F113" t="n">
         <v>8</v>
       </c>
-      <c r="J113" t="n">
+      <c r="G113" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H113" t="n">
+        <v>7</v>
+      </c>
+      <c r="M113" t="n">
         <v>7</v>
       </c>
       <c r="O113" t="n">
         <v>1</v>
       </c>
-      <c r="S113" t="n">
+      <c r="P113" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>1</v>
+      </c>
+      <c r="V113" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z113" t="n">
         <v>1</v>
       </c>
       <c r="AF113" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG113" t="inlineStr">
         <is>
@@ -8167,7 +8191,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Ingeniería genética y ADN recombinante</t>
+          <t>Inmunidad adaptativa</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -8178,27 +8202,15 @@
       <c r="C114" t="n">
         <v>9</v>
       </c>
-      <c r="F114" t="n">
-        <v>8</v>
-      </c>
       <c r="G114" t="n">
         <v>8.5</v>
       </c>
-      <c r="H114" t="n">
-        <v>7</v>
-      </c>
       <c r="M114" t="n">
         <v>7</v>
       </c>
-      <c r="O114" t="n">
-        <v>1</v>
-      </c>
       <c r="P114" t="n">
         <v>1</v>
       </c>
-      <c r="Q114" t="n">
-        <v>1</v>
-      </c>
       <c r="V114" t="n">
         <v>1</v>
       </c>
@@ -8206,7 +8218,7 @@
         <v>1</v>
       </c>
       <c r="AF114" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG114" t="inlineStr">
         <is>
@@ -8222,7 +8234,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Inmunidad adaptativa</t>
+          <t>Inmunidad innata</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8245,9 +8257,6 @@
       <c r="V115" t="n">
         <v>1</v>
       </c>
-      <c r="Z115" t="n">
-        <v>1</v>
-      </c>
       <c r="AF115" t="n">
         <v>10</v>
       </c>
@@ -8265,7 +8274,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Inmunidad innata</t>
+          <t>Nutrición mineral de las plantas</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -8274,22 +8283,28 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F116" t="n">
+        <v>5</v>
       </c>
       <c r="G116" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M116" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="I116" t="n">
+        <v>4</v>
+      </c>
+      <c r="O116" t="n">
+        <v>1</v>
       </c>
       <c r="P116" t="n">
         <v>1</v>
       </c>
-      <c r="V116" t="n">
+      <c r="R116" t="n">
         <v>1</v>
       </c>
       <c r="AF116" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG116" t="inlineStr">
         <is>
@@ -8305,7 +8320,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Nutrición mineral de las plantas</t>
+          <t>Presión y flujo de fluidos en los seres vivos</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -8316,22 +8331,16 @@
       <c r="C117" t="n">
         <v>11</v>
       </c>
-      <c r="F117" t="n">
-        <v>5</v>
-      </c>
-      <c r="G117" t="n">
-        <v>2</v>
-      </c>
-      <c r="I117" t="n">
-        <v>4</v>
-      </c>
-      <c r="O117" t="n">
-        <v>1</v>
-      </c>
-      <c r="P117" t="n">
-        <v>1</v>
-      </c>
-      <c r="R117" t="n">
+      <c r="H117" t="n">
+        <v>7</v>
+      </c>
+      <c r="M117" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>1</v>
+      </c>
+      <c r="V117" t="n">
         <v>1</v>
       </c>
       <c r="AF117" t="n">
@@ -8351,7 +8360,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Presión y flujo de fluidos en los seres vivos</t>
+          <t>Proteínas: estructura y función</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -8360,26 +8369,23 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>11</v>
-      </c>
-      <c r="H118" t="n">
-        <v>7</v>
-      </c>
-      <c r="M118" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q118" t="n">
-        <v>1</v>
-      </c>
-      <c r="V118" t="n">
+        <v>6</v>
+      </c>
+      <c r="D118" t="n">
+        <v>6</v>
+      </c>
+      <c r="G118" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="P118" t="n">
         <v>1</v>
       </c>
       <c r="AF118" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG118" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH118" t="inlineStr">
@@ -8391,7 +8397,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Proteínas: estructura y función</t>
+          <t>Regulación de la expresión génica</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -8400,14 +8406,17 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6</v>
-      </c>
-      <c r="D119" t="n">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="F119" t="n">
+        <v>8</v>
       </c>
       <c r="G119" t="n">
         <v>8.5</v>
       </c>
+      <c r="O119" t="n">
+        <v>1</v>
+      </c>
       <c r="P119" t="n">
         <v>1</v>
       </c>
@@ -8416,7 +8425,7 @@
       </c>
       <c r="AG119" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH119" t="inlineStr">
@@ -8428,7 +8437,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Regulación de la expresión génica</t>
+          <t>Relación superficie-volumen</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -8437,7 +8446,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F120" t="n">
         <v>8</v>
@@ -8445,14 +8454,32 @@
       <c r="G120" t="n">
         <v>8.5</v>
       </c>
+      <c r="J120" t="n">
+        <v>7</v>
+      </c>
+      <c r="K120" t="n">
+        <v>7</v>
+      </c>
+      <c r="L120" t="n">
+        <v>7.5</v>
+      </c>
       <c r="O120" t="n">
         <v>1</v>
       </c>
       <c r="P120" t="n">
         <v>1</v>
       </c>
+      <c r="S120" t="n">
+        <v>1</v>
+      </c>
+      <c r="T120" t="n">
+        <v>1</v>
+      </c>
+      <c r="U120" t="n">
+        <v>1</v>
+      </c>
       <c r="AF120" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG120" t="inlineStr">
         <is>
@@ -8461,14 +8488,14 @@
       </c>
       <c r="AH120" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Relación superficie-volumen</t>
+          <t>Relaciones intraespecíficas</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -8477,56 +8504,35 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>10</v>
-      </c>
-      <c r="F121" t="n">
-        <v>8</v>
-      </c>
-      <c r="G121" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J121" t="n">
-        <v>7</v>
-      </c>
-      <c r="K121" t="n">
-        <v>7</v>
-      </c>
-      <c r="L121" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="O121" t="n">
-        <v>1</v>
-      </c>
-      <c r="P121" t="n">
-        <v>1</v>
-      </c>
-      <c r="S121" t="n">
-        <v>1</v>
-      </c>
-      <c r="T121" t="n">
-        <v>1</v>
-      </c>
-      <c r="U121" t="n">
+        <v>7</v>
+      </c>
+      <c r="D121" t="n">
+        <v>7</v>
+      </c>
+      <c r="M121" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="V121" t="n">
         <v>1</v>
       </c>
       <c r="AF121" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG121" t="inlineStr">
         <is>
+          <t>sin_referente</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
           <t>posterior</t>
-        </is>
-      </c>
-      <c r="AH121" t="inlineStr">
-        <is>
-          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Relaciones intraespecíficas</t>
+          <t>Sistema inmunitario</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -8535,23 +8541,35 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>7</v>
-      </c>
-      <c r="D122" t="n">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="F122" t="n">
+        <v>8</v>
+      </c>
+      <c r="G122" t="n">
+        <v>8.5</v>
       </c>
       <c r="M122" t="n">
-        <v>4.5</v>
+        <v>7</v>
+      </c>
+      <c r="O122" t="n">
+        <v>1</v>
+      </c>
+      <c r="P122" t="n">
+        <v>1</v>
       </c>
       <c r="V122" t="n">
         <v>1</v>
       </c>
+      <c r="Z122" t="n">
+        <v>1</v>
+      </c>
       <c r="AF122" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG122" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH122" t="inlineStr">
@@ -8563,7 +8581,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Sistema inmunitario</t>
+          <t>Termorregulación</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -8572,31 +8590,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F123" t="n">
         <v>8</v>
       </c>
-      <c r="G123" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M123" t="n">
-        <v>7</v>
-      </c>
       <c r="O123" t="n">
         <v>1</v>
       </c>
-      <c r="P123" t="n">
-        <v>1</v>
-      </c>
-      <c r="V123" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z123" t="n">
-        <v>1</v>
-      </c>
       <c r="AF123" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG123" t="inlineStr">
         <is>
@@ -8612,7 +8615,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Termorregulación</t>
+          <t>Virus</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -8621,20 +8624,41 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>10</v>
+        <v>3</v>
+      </c>
+      <c r="D124" t="n">
+        <v>3</v>
       </c>
       <c r="F124" t="n">
         <v>8</v>
       </c>
+      <c r="G124" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H124" t="n">
+        <v>4</v>
+      </c>
+      <c r="L124" t="n">
+        <v>7.5</v>
+      </c>
       <c r="O124" t="n">
         <v>1</v>
       </c>
+      <c r="P124" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>1</v>
+      </c>
+      <c r="U124" t="n">
+        <v>1</v>
+      </c>
       <c r="AF124" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG124" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH124" t="inlineStr">
@@ -8646,59 +8670,44 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Virus</t>
+          <t>Acervo génico y frecuencias alélicas</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>9</v>
-      </c>
-      <c r="F125" t="n">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="D125" t="n">
+        <v>7</v>
       </c>
       <c r="G125" t="n">
         <v>8.5</v>
       </c>
-      <c r="H125" t="n">
-        <v>4</v>
-      </c>
-      <c r="L125" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="O125" t="n">
-        <v>1</v>
-      </c>
       <c r="P125" t="n">
         <v>1</v>
       </c>
-      <c r="Q125" t="n">
-        <v>1</v>
-      </c>
-      <c r="U125" t="n">
-        <v>1</v>
-      </c>
       <c r="AF125" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AG125" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH125" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Acervo génico y frecuencias alélicas</t>
+          <t>ATP y energía en los sistemas vivos</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -8707,19 +8716,31 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D126" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G126" t="n">
-        <v>8.5</v>
+        <v>6</v>
+      </c>
+      <c r="H126" t="n">
+        <v>7</v>
+      </c>
+      <c r="J126" t="n">
+        <v>7</v>
       </c>
       <c r="P126" t="n">
         <v>1</v>
       </c>
+      <c r="Q126" t="n">
+        <v>1</v>
+      </c>
+      <c r="S126" t="n">
+        <v>1</v>
+      </c>
       <c r="AF126" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG126" t="inlineStr">
         <is>
@@ -8728,14 +8749,14 @@
       </c>
       <c r="AH126" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ATP y energía en los sistemas vivos</t>
+          <t>Atributos de las poblaciones</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -8744,31 +8765,37 @@
         </is>
       </c>
       <c r="C127" t="n">
+        <v>7</v>
+      </c>
+      <c r="D127" t="n">
+        <v>7</v>
+      </c>
+      <c r="F127" t="n">
+        <v>8</v>
+      </c>
+      <c r="G127" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L127" t="n">
         <v>6</v>
       </c>
-      <c r="D127" t="n">
-        <v>6</v>
-      </c>
-      <c r="G127" t="n">
-        <v>6</v>
-      </c>
-      <c r="H127" t="n">
-        <v>7</v>
-      </c>
-      <c r="J127" t="n">
-        <v>7</v>
+      <c r="M127" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O127" t="n">
+        <v>1</v>
       </c>
       <c r="P127" t="n">
         <v>1</v>
       </c>
-      <c r="Q127" t="n">
-        <v>1</v>
-      </c>
-      <c r="S127" t="n">
+      <c r="U127" t="n">
+        <v>1</v>
+      </c>
+      <c r="V127" t="n">
         <v>1</v>
       </c>
       <c r="AF127" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG127" t="inlineStr">
         <is>
@@ -8784,7 +8811,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Atributos de las poblaciones</t>
+          <t>Biomas y clasificación de ambientes</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -8793,37 +8820,25 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D128" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F128" t="n">
         <v>8</v>
       </c>
-      <c r="G128" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="L128" t="n">
-        <v>6</v>
-      </c>
-      <c r="M128" t="n">
-        <v>4.5</v>
+      <c r="H128" t="n">
+        <v>3</v>
       </c>
       <c r="O128" t="n">
         <v>1</v>
       </c>
-      <c r="P128" t="n">
-        <v>1</v>
-      </c>
-      <c r="U128" t="n">
-        <v>1</v>
-      </c>
-      <c r="V128" t="n">
+      <c r="Q128" t="n">
         <v>1</v>
       </c>
       <c r="AF128" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AG128" t="inlineStr">
         <is>
@@ -8832,14 +8847,14 @@
       </c>
       <c r="AH128" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Biomas y clasificación de ambientes</t>
+          <t>Célula procariota y eucariota</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -8848,25 +8863,25 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D129" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F129" t="n">
         <v>8</v>
       </c>
-      <c r="H129" t="n">
-        <v>3</v>
+      <c r="G129" t="n">
+        <v>8.5</v>
       </c>
       <c r="O129" t="n">
         <v>1</v>
       </c>
-      <c r="Q129" t="n">
+      <c r="P129" t="n">
         <v>1</v>
       </c>
       <c r="AF129" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AG129" t="inlineStr">
         <is>
@@ -8882,7 +8897,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Célula procariota y eucariota</t>
+          <t>Conservación e inocuidad de los alimentos</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -8891,25 +8906,25 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D130" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F130" t="n">
         <v>8</v>
       </c>
-      <c r="G130" t="n">
-        <v>8.5</v>
+      <c r="H130" t="n">
+        <v>2</v>
       </c>
       <c r="O130" t="n">
         <v>1</v>
       </c>
-      <c r="P130" t="n">
+      <c r="Q130" t="n">
         <v>1</v>
       </c>
       <c r="AF130" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="AG130" t="inlineStr">
         <is>
@@ -8925,7 +8940,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Conservación e inocuidad de los alimentos</t>
+          <t>Ecosistemas acuáticos y marinos</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -8934,25 +8949,25 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
-        <v>2</v>
-      </c>
-      <c r="F131" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
-      </c>
-      <c r="O131" t="n">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="J131" t="n">
+        <v>2.5</v>
       </c>
       <c r="Q131" t="n">
         <v>1</v>
       </c>
+      <c r="S131" t="n">
+        <v>1</v>
+      </c>
       <c r="AF131" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AG131" t="inlineStr">
         <is>
@@ -8968,7 +8983,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Ecosistemas acuáticos y marinos</t>
+          <t>Ecosistemas naturales, rurales y urbanos</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -8977,25 +8992,25 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D132" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H132" t="n">
         <v>7</v>
       </c>
-      <c r="J132" t="n">
+      <c r="M132" t="n">
         <v>2.5</v>
       </c>
       <c r="Q132" t="n">
         <v>1</v>
       </c>
-      <c r="S132" t="n">
+      <c r="V132" t="n">
         <v>1</v>
       </c>
       <c r="AF132" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG132" t="inlineStr">
         <is>
@@ -9011,7 +9026,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Ecosistemas naturales, rurales y urbanos</t>
+          <t>Estrategias reproductivas y supervivencia de la descendencia</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -9020,25 +9035,43 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E133" t="n">
+        <v>8</v>
+      </c>
+      <c r="F133" t="n">
+        <v>8</v>
       </c>
       <c r="H133" t="n">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="L133" t="n">
+        <v>6</v>
       </c>
       <c r="M133" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
+      </c>
+      <c r="N133" t="n">
+        <v>1</v>
+      </c>
+      <c r="O133" t="n">
+        <v>1</v>
       </c>
       <c r="Q133" t="n">
         <v>1</v>
       </c>
+      <c r="U133" t="n">
+        <v>1</v>
+      </c>
       <c r="V133" t="n">
         <v>1</v>
       </c>
       <c r="AF133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG133" t="inlineStr">
         <is>
@@ -9047,14 +9080,14 @@
       </c>
       <c r="AH133" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Estrategias reproductivas y supervivencia de la descendencia</t>
+          <t>Estructura del ADN</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -9063,43 +9096,22 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D134" t="n">
-        <v>3</v>
-      </c>
-      <c r="E134" t="n">
-        <v>8</v>
-      </c>
-      <c r="F134" t="n">
-        <v>8</v>
-      </c>
-      <c r="H134" t="n">
-        <v>3</v>
-      </c>
-      <c r="L134" t="n">
         <v>6</v>
       </c>
-      <c r="M134" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N134" t="n">
-        <v>1</v>
-      </c>
-      <c r="O134" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q134" t="n">
-        <v>1</v>
-      </c>
-      <c r="U134" t="n">
-        <v>1</v>
-      </c>
-      <c r="V134" t="n">
+      <c r="G134" t="n">
+        <v>6</v>
+      </c>
+      <c r="P134" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z134" t="n">
         <v>1</v>
       </c>
       <c r="AF134" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG134" t="inlineStr">
         <is>
@@ -9108,14 +9120,14 @@
       </c>
       <c r="AH134" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Estructura del ADN</t>
+          <t>Fermentación y respiración anaerobia</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -9124,22 +9136,25 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G135" t="n">
         <v>6</v>
       </c>
+      <c r="M135" t="n">
+        <v>7</v>
+      </c>
       <c r="P135" t="n">
         <v>1</v>
       </c>
-      <c r="Z135" t="n">
+      <c r="V135" t="n">
         <v>1</v>
       </c>
       <c r="AF135" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG135" t="inlineStr">
         <is>
@@ -9155,7 +9170,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Fermentación y respiración anaerobia</t>
+          <t>Filogenia y parentesco evolutivo</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -9164,25 +9179,25 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D136" t="n">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="F136" t="n">
+        <v>8</v>
       </c>
       <c r="G136" t="n">
-        <v>6</v>
-      </c>
-      <c r="M136" t="n">
-        <v>7</v>
+        <v>8.5</v>
+      </c>
+      <c r="O136" t="n">
+        <v>1</v>
       </c>
       <c r="P136" t="n">
         <v>1</v>
       </c>
-      <c r="V136" t="n">
-        <v>1</v>
-      </c>
       <c r="AF136" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AG136" t="inlineStr">
         <is>
@@ -9198,7 +9213,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Filogenia y parentesco evolutivo</t>
+          <t>Mecanismos de microevolución</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -9215,13 +9230,10 @@
       <c r="F137" t="n">
         <v>8</v>
       </c>
-      <c r="G137" t="n">
-        <v>8.5</v>
-      </c>
       <c r="O137" t="n">
         <v>1</v>
       </c>
-      <c r="P137" t="n">
+      <c r="Z137" t="n">
         <v>1</v>
       </c>
       <c r="AF137" t="n">
@@ -9241,7 +9253,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Mecanismos de microevolución</t>
+          <t>Medidas de biodiversidad</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -9255,13 +9267,10 @@
       <c r="D138" t="n">
         <v>7</v>
       </c>
-      <c r="F138" t="n">
-        <v>8</v>
-      </c>
-      <c r="O138" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z138" t="n">
+      <c r="H138" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q138" t="n">
         <v>1</v>
       </c>
       <c r="AF138" t="n">
@@ -9281,7 +9290,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Medidas de biodiversidad</t>
+          <t>Membrana celular</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -9290,19 +9299,28 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D139" t="n">
-        <v>7</v>
-      </c>
-      <c r="H139" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q139" t="n">
+        <v>6</v>
+      </c>
+      <c r="G139" t="n">
+        <v>6</v>
+      </c>
+      <c r="K139" t="n">
+        <v>7</v>
+      </c>
+      <c r="P139" t="n">
+        <v>1</v>
+      </c>
+      <c r="T139" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z139" t="n">
         <v>1</v>
       </c>
       <c r="AF139" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG139" t="inlineStr">
         <is>
@@ -9318,7 +9336,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Membrana celular</t>
+          <t>Modelos ecológicos basados en muestreo</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -9327,28 +9345,19 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D140" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G140" t="n">
-        <v>6</v>
-      </c>
-      <c r="K140" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="P140" t="n">
         <v>1</v>
       </c>
-      <c r="T140" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z140" t="n">
-        <v>1</v>
-      </c>
       <c r="AF140" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG140" t="inlineStr">
         <is>
@@ -9364,7 +9373,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Modelos ecológicos basados en muestreo</t>
+          <t>Mutaciones</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -9381,7 +9390,16 @@
       <c r="G141" t="n">
         <v>8.5</v>
       </c>
+      <c r="M141" t="n">
+        <v>7</v>
+      </c>
       <c r="P141" t="n">
+        <v>1</v>
+      </c>
+      <c r="V141" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z141" t="n">
         <v>1</v>
       </c>
       <c r="AF141" t="n">
@@ -9401,7 +9419,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Mutaciones</t>
+          <t>Nicho ecológico y exclusión competitiva</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -9410,28 +9428,19 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D142" t="n">
-        <v>7</v>
-      </c>
-      <c r="G142" t="n">
-        <v>8.5</v>
+        <v>4</v>
       </c>
       <c r="M142" t="n">
         <v>7</v>
       </c>
-      <c r="P142" t="n">
-        <v>1</v>
-      </c>
       <c r="V142" t="n">
         <v>1</v>
       </c>
-      <c r="Z142" t="n">
-        <v>1</v>
-      </c>
       <c r="AF142" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AG142" t="inlineStr">
         <is>
@@ -9447,7 +9456,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Nicho ecológico y exclusión competitiva</t>
+          <t>Organelos de la célula eucariota</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -9456,19 +9465,37 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D143" t="n">
-        <v>4</v>
-      </c>
-      <c r="M143" t="n">
-        <v>7</v>
-      </c>
-      <c r="V143" t="n">
+        <v>6</v>
+      </c>
+      <c r="E143" t="n">
+        <v>7</v>
+      </c>
+      <c r="G143" t="n">
+        <v>6</v>
+      </c>
+      <c r="K143" t="n">
+        <v>7</v>
+      </c>
+      <c r="L143" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="N143" t="n">
+        <v>1</v>
+      </c>
+      <c r="P143" t="n">
+        <v>1</v>
+      </c>
+      <c r="T143" t="n">
+        <v>1</v>
+      </c>
+      <c r="U143" t="n">
         <v>1</v>
       </c>
       <c r="AF143" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AG143" t="inlineStr">
         <is>
@@ -9477,14 +9504,14 @@
       </c>
       <c r="AH143" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Organelos de la célula eucariota</t>
+          <t>Osmorregulación y equilibrio hídrico</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -9493,37 +9520,13 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
-      </c>
-      <c r="E144" t="n">
-        <v>7</v>
-      </c>
-      <c r="G144" t="n">
-        <v>6</v>
-      </c>
-      <c r="K144" t="n">
-        <v>7</v>
-      </c>
-      <c r="L144" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="N144" t="n">
-        <v>1</v>
-      </c>
-      <c r="P144" t="n">
-        <v>1</v>
-      </c>
-      <c r="T144" t="n">
-        <v>1</v>
-      </c>
-      <c r="U144" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AF144" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AG144" t="inlineStr">
         <is>
@@ -9532,14 +9535,14 @@
       </c>
       <c r="AH144" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Osmorregulación y equilibrio hídrico</t>
+          <t>PCR y electroforesis en gel</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -9553,8 +9556,14 @@
       <c r="D145" t="n">
         <v>7</v>
       </c>
+      <c r="H145" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>1</v>
+      </c>
       <c r="AF145" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AG145" t="inlineStr">
         <is>
@@ -9570,7 +9579,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>PCR y electroforesis en gel</t>
+          <t>Replicación del ADN</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -9583,12 +9592,6 @@
       </c>
       <c r="D146" t="n">
         <v>7</v>
-      </c>
-      <c r="H146" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q146" t="n">
-        <v>1</v>
       </c>
       <c r="AF146" t="n">
         <v>7</v>
@@ -9607,7 +9610,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Replicación del ADN</t>
+          <t>Selección artificial</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -9620,6 +9623,18 @@
       </c>
       <c r="D147" t="n">
         <v>7</v>
+      </c>
+      <c r="G147" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="M147" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="P147" t="n">
+        <v>1</v>
+      </c>
+      <c r="V147" t="n">
+        <v>1</v>
       </c>
       <c r="AF147" t="n">
         <v>7</v>
@@ -9638,7 +9653,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Selección artificial</t>
+          <t>Síntesis de proteínas</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -9652,16 +9667,7 @@
       <c r="D148" t="n">
         <v>7</v>
       </c>
-      <c r="G148" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M148" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="P148" t="n">
-        <v>1</v>
-      </c>
-      <c r="V148" t="n">
+      <c r="Z148" t="n">
         <v>1</v>
       </c>
       <c r="AF148" t="n">
@@ -9681,7 +9687,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Síntesis de proteínas</t>
+          <t>Sucesión ecológica</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -9695,7 +9701,16 @@
       <c r="D149" t="n">
         <v>7</v>
       </c>
-      <c r="Z149" t="n">
+      <c r="K149" t="n">
+        <v>5</v>
+      </c>
+      <c r="M149" t="n">
+        <v>7</v>
+      </c>
+      <c r="T149" t="n">
+        <v>1</v>
+      </c>
+      <c r="V149" t="n">
         <v>1</v>
       </c>
       <c r="AF149" t="n">
@@ -9715,7 +9730,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Sucesión ecológica</t>
+          <t>Transporte activo y endocitosis</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -9724,25 +9739,19 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D150" t="n">
-        <v>7</v>
-      </c>
-      <c r="K150" t="n">
-        <v>5</v>
-      </c>
-      <c r="M150" t="n">
-        <v>7</v>
-      </c>
-      <c r="T150" t="n">
-        <v>1</v>
-      </c>
-      <c r="V150" t="n">
+        <v>6</v>
+      </c>
+      <c r="G150" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="P150" t="n">
         <v>1</v>
       </c>
       <c r="AF150" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG150" t="inlineStr">
         <is>
@@ -9758,7 +9767,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Transporte activo y endocitosis</t>
+          <t>Tropismos y hormonas vegetales</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -9767,19 +9776,19 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
-        <v>6</v>
-      </c>
-      <c r="G151" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="P151" t="n">
+        <v>3</v>
+      </c>
+      <c r="K151" t="n">
+        <v>2</v>
+      </c>
+      <c r="T151" t="n">
         <v>1</v>
       </c>
       <c r="AF151" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG151" t="inlineStr">
         <is>
@@ -9787,43 +9796,6 @@
         </is>
       </c>
       <c r="AH151" t="inlineStr">
-        <is>
-          <t>sin_referente</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Tropismos y hormonas vegetales</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>sin_referente</t>
-        </is>
-      </c>
-      <c r="C152" t="n">
-        <v>3</v>
-      </c>
-      <c r="D152" t="n">
-        <v>3</v>
-      </c>
-      <c r="K152" t="n">
-        <v>2</v>
-      </c>
-      <c r="T152" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF152" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG152" t="inlineStr">
-        <is>
-          <t>sin_referente</t>
-        </is>
-      </c>
-      <c r="AH152" t="inlineStr">
         <is>
           <t>sin_referente</t>
         </is>
@@ -9840,7 +9812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -16195,48 +16167,6 @@
       </c>
       <c r="J151">
         <f>Datos!B151</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152">
-        <f>Datos!A152</f>
-        <v/>
-      </c>
-      <c r="B152">
-        <f>IF(Datos!C152="","",Datos!C152)</f>
-        <v/>
-      </c>
-      <c r="C152">
-        <f>COUNT(Datos!E152:M152)</f>
-        <v/>
-      </c>
-      <c r="D152">
-        <f>IF(C152=0,"",MEDIAN(Datos!E152:M152))</f>
-        <v/>
-      </c>
-      <c r="E152">
-        <f>COUNT(Datos!W152:AE152)</f>
-        <v/>
-      </c>
-      <c r="F152">
-        <f>IF(OR(B152="",D152=""),"",B152-D152)</f>
-        <v/>
-      </c>
-      <c r="G152">
-        <f>IF(Datos!D152="","",Datos!D152)</f>
-        <v/>
-      </c>
-      <c r="H152">
-        <f>COUNT(Datos!N152:V152)</f>
-        <v/>
-      </c>
-      <c r="I152">
-        <f>IF(B152="",IF(C152&gt;=5,"falta en SV",""),IF(G152="",IF(B152&gt;8,IF(C152&gt;=5,"SV tarde","despues del tramo"),IF(H152&gt;=5,"no retomado en 2-8","previo")),IF(B152&lt;2,"retomado",IF(AND(C152&lt;=1,E152&gt;=3),"solo especializacion",IF(F152="","coherente",IF(F152&lt;=-1.5,"SV adelantado",IF(F152&gt;=2,"SV tarde","coherente")))))))</f>
-        <v/>
-      </c>
-      <c r="J152">
-        <f>Datos!B152</f>
         <v/>
       </c>
     </row>
@@ -16276,7 +16206,7 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF(Datos!B2:B152,A2)</f>
+        <f>COUNTIF(Datos!B2:B151,A2)</f>
         <v/>
       </c>
     </row>
@@ -16287,7 +16217,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF(Datos!B2:B152,A3)</f>
+        <f>COUNTIF(Datos!B2:B151,A3)</f>
         <v/>
       </c>
     </row>
@@ -16298,7 +16228,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Datos!B2:B152,A4)</f>
+        <f>COUNTIF(Datos!B2:B151,A4)</f>
         <v/>
       </c>
     </row>
@@ -16309,7 +16239,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Datos!B2:B152,A5)</f>
+        <f>COUNTIF(Datos!B2:B151,A5)</f>
         <v/>
       </c>
     </row>
@@ -16320,7 +16250,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Datos!B2:B152,A6)</f>
+        <f>COUNTIF(Datos!B2:B151,A6)</f>
         <v/>
       </c>
     </row>
@@ -16331,7 +16261,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF(Datos!B2:B152,A7)</f>
+        <f>COUNTIF(Datos!B2:B151,A7)</f>
         <v/>
       </c>
     </row>
@@ -16342,7 +16272,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF(Datos!B2:B152,A8)</f>
+        <f>COUNTIF(Datos!B2:B151,A8)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(panel): serie v3 aplicada; el contraste queda sin inciertos sobre la V3
- 87 expedientes de la serie v3 resueltos y aplicados (38 inciertos nuevos
  y 49 clases re-decididas con la V3; cambian, entre otras, biotecnología
  vegetal, espectrometría, técnicas de estructura, lípidos, ley de Ohm y
  modelo estándar). Ningún concepto incierto en 2.°–8.° ni en 9.°–11.°.
- Refuerzos de Física y Química 9.°–11.°, serie a: 13 para inyectar (12
  notas y 1 fila) y 3 descartes, unidos en refuerzos.json para el panel.
- Serie b (8 candidatos que esperaban la re-decisión) en redacción; lotes
  del bucle (refutador, serie v3) y de la revisión del panel preparados.
- Snapshot de Física y Química 9.°–11.° actualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_biologia.xlsx
+++ b/internacional/2_8/Contraste_biologia.xlsx
@@ -2518,7 +2518,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Biotecnología vegetal y agroindustria</t>
+          <t>Cadena alimentaria</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2527,19 +2527,40 @@
         </is>
       </c>
       <c r="C30" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>3</v>
+      </c>
+      <c r="I30" t="n">
+        <v>5</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K30" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" t="n">
         <v>6</v>
       </c>
-      <c r="D30" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" t="n">
-        <v>8</v>
-      </c>
-      <c r="G30" t="n">
-        <v>8.5</v>
-      </c>
       <c r="M30" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1</v>
       </c>
       <c r="O30" t="n">
         <v>1</v>
@@ -2547,27 +2568,42 @@
       <c r="P30" t="n">
         <v>1</v>
       </c>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="n">
+        <v>1</v>
+      </c>
+      <c r="T30" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" t="n">
+        <v>1</v>
+      </c>
       <c r="V30" t="n">
         <v>1</v>
       </c>
       <c r="AF30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cadena alimentaria</t>
+          <t>Cambio climático y seres vivos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2576,31 +2612,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G31" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
-      </c>
-      <c r="I31" t="n">
+        <v>7</v>
+      </c>
+      <c r="K31" t="n">
         <v>5</v>
-      </c>
-      <c r="J31" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K31" t="n">
-        <v>2</v>
       </c>
       <c r="L31" t="n">
         <v>6</v>
@@ -2608,24 +2632,12 @@
       <c r="M31" t="n">
         <v>4.5</v>
       </c>
-      <c r="N31" t="n">
-        <v>1</v>
-      </c>
       <c r="O31" t="n">
         <v>1</v>
       </c>
-      <c r="P31" t="n">
-        <v>1</v>
-      </c>
       <c r="Q31" t="n">
         <v>1</v>
       </c>
-      <c r="R31" t="n">
-        <v>1</v>
-      </c>
-      <c r="S31" t="n">
-        <v>1</v>
-      </c>
       <c r="T31" t="n">
         <v>1</v>
       </c>
@@ -2636,7 +2648,7 @@
         <v>1</v>
       </c>
       <c r="AF31" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="AG31" t="inlineStr">
         <is>
@@ -2645,14 +2657,14 @@
       </c>
       <c r="AH31" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambio climático y seres vivos</t>
+          <t>Célula animal y célula vegetal</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2661,32 +2673,56 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="n">
         <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>8</v>
       </c>
+      <c r="G32" t="n">
+        <v>6</v>
+      </c>
       <c r="H32" t="n">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>7</v>
+      </c>
+      <c r="J32" t="n">
+        <v>4.5</v>
       </c>
       <c r="K32" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L32" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="M32" t="n">
-        <v>4.5</v>
+        <v>7</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1</v>
       </c>
       <c r="O32" t="n">
         <v>1</v>
       </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
       <c r="Q32" t="n">
         <v>1</v>
       </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>1</v>
+      </c>
       <c r="T32" t="n">
         <v>1</v>
       </c>
@@ -2697,7 +2733,7 @@
         <v>1</v>
       </c>
       <c r="AF32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG32" t="inlineStr">
         <is>
@@ -3913,7 +3949,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Estructuras del cuerpo animal y su función</t>
+          <t>Estructuras celulares básicas</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3922,37 +3958,37 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F51" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I51" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J51" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="K51" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L51" t="n">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="M51" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="N51" t="n">
         <v>1</v>
@@ -3985,7 +4021,7 @@
         <v>1</v>
       </c>
       <c r="AF51" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
@@ -3994,14 +4030,14 @@
       </c>
       <c r="AH51" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Extinción de especies</t>
+          <t>Estructuras del cuerpo animal y su función</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4010,28 +4046,40 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
       </c>
       <c r="F52" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G52" t="n">
         <v>2</v>
       </c>
       <c r="H52" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" t="n">
+        <v>2.5</v>
       </c>
       <c r="K52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M52" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1</v>
       </c>
       <c r="O52" t="n">
         <v>1</v>
@@ -4042,6 +4090,12 @@
       <c r="Q52" t="n">
         <v>1</v>
       </c>
+      <c r="R52" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1</v>
+      </c>
       <c r="T52" t="n">
         <v>1</v>
       </c>
@@ -4051,8 +4105,11 @@
       <c r="V52" t="n">
         <v>1</v>
       </c>
+      <c r="Z52" t="n">
+        <v>1</v>
+      </c>
       <c r="AF52" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AG52" t="inlineStr">
         <is>
@@ -4068,7 +4125,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Factores bióticos y abióticos</t>
+          <t>Extinción de especies</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4077,68 +4134,50 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" t="n">
         <v>5</v>
       </c>
       <c r="F53" t="n">
+        <v>8</v>
+      </c>
+      <c r="G53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H53" t="n">
         <v>5</v>
       </c>
-      <c r="G53" t="n">
-        <v>2</v>
-      </c>
-      <c r="H53" t="n">
-        <v>2</v>
-      </c>
-      <c r="I53" t="n">
+      <c r="K53" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" t="n">
+        <v>6</v>
+      </c>
+      <c r="M53" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="O53" t="n">
+        <v>1</v>
+      </c>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>1</v>
+      </c>
+      <c r="T53" t="n">
+        <v>1</v>
+      </c>
+      <c r="U53" t="n">
+        <v>1</v>
+      </c>
+      <c r="V53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF53" t="n">
         <v>5</v>
       </c>
-      <c r="J53" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K53" t="n">
-        <v>2</v>
-      </c>
-      <c r="L53" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M53" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N53" t="n">
-        <v>1</v>
-      </c>
-      <c r="O53" t="n">
-        <v>1</v>
-      </c>
-      <c r="P53" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>1</v>
-      </c>
-      <c r="R53" t="n">
-        <v>1</v>
-      </c>
-      <c r="S53" t="n">
-        <v>1</v>
-      </c>
-      <c r="T53" t="n">
-        <v>1</v>
-      </c>
-      <c r="U53" t="n">
-        <v>1</v>
-      </c>
-      <c r="V53" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF53" t="n">
-        <v>4</v>
-      </c>
       <c r="AG53" t="inlineStr">
         <is>
           <t>alineado</t>
@@ -4146,14 +4185,14 @@
       </c>
       <c r="AH53" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Factores limitantes de las poblaciones</t>
+          <t>Factores bióticos y abióticos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4162,28 +4201,37 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G54" t="n">
-        <v>8.5</v>
+        <v>2</v>
+      </c>
+      <c r="H54" t="n">
+        <v>2</v>
+      </c>
+      <c r="I54" t="n">
+        <v>5</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2.5</v>
       </c>
       <c r="K54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L54" t="n">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="M54" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="N54" t="n">
         <v>1</v>
@@ -4194,6 +4242,15 @@
       <c r="P54" t="n">
         <v>1</v>
       </c>
+      <c r="Q54" t="n">
+        <v>1</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="n">
+        <v>1</v>
+      </c>
       <c r="T54" t="n">
         <v>1</v>
       </c>
@@ -4204,11 +4261,11 @@
         <v>1</v>
       </c>
       <c r="AF54" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH54" t="inlineStr">
@@ -4220,7 +4277,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fecundación y desarrollo embrionario</t>
+          <t>Factores limitantes de las poblaciones</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4229,28 +4286,31 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D55" t="n">
+        <v>7</v>
+      </c>
+      <c r="E55" t="n">
         <v>6</v>
       </c>
       <c r="F55" t="n">
         <v>8</v>
       </c>
       <c r="G55" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3</v>
+      </c>
+      <c r="L55" t="n">
         <v>6</v>
       </c>
-      <c r="H55" t="n">
-        <v>7</v>
-      </c>
-      <c r="I55" t="n">
-        <v>4</v>
-      </c>
-      <c r="J55" t="n">
-        <v>7</v>
-      </c>
-      <c r="L55" t="n">
-        <v>5</v>
+      <c r="M55" t="n">
+        <v>7</v>
+      </c>
+      <c r="N55" t="n">
+        <v>1</v>
       </c>
       <c r="O55" t="n">
         <v>1</v>
@@ -4258,39 +4318,33 @@
       <c r="P55" t="n">
         <v>1</v>
       </c>
-      <c r="Q55" t="n">
-        <v>1</v>
-      </c>
-      <c r="R55" t="n">
-        <v>1</v>
-      </c>
-      <c r="S55" t="n">
+      <c r="T55" t="n">
         <v>1</v>
       </c>
       <c r="U55" t="n">
         <v>1</v>
       </c>
-      <c r="Z55" t="n">
+      <c r="V55" t="n">
         <v>1</v>
       </c>
       <c r="AF55" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH55" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Flujo de energía y pirámides ecológicas</t>
+          <t>Fecundación y desarrollo embrionario</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4299,49 +4353,52 @@
         </is>
       </c>
       <c r="C56" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" t="n">
+        <v>6</v>
+      </c>
+      <c r="F56" t="n">
+        <v>8</v>
+      </c>
+      <c r="G56" t="n">
+        <v>6</v>
+      </c>
+      <c r="H56" t="n">
+        <v>7</v>
+      </c>
+      <c r="I56" t="n">
+        <v>4</v>
+      </c>
+      <c r="J56" t="n">
+        <v>7</v>
+      </c>
+      <c r="L56" t="n">
         <v>5</v>
       </c>
-      <c r="D56" t="n">
-        <v>5</v>
-      </c>
-      <c r="E56" t="n">
+      <c r="O56" t="n">
+        <v>1</v>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>1</v>
+      </c>
+      <c r="R56" t="n">
+        <v>1</v>
+      </c>
+      <c r="S56" t="n">
+        <v>1</v>
+      </c>
+      <c r="U56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF56" t="n">
         <v>6</v>
-      </c>
-      <c r="G56" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H56" t="n">
-        <v>5</v>
-      </c>
-      <c r="K56" t="n">
-        <v>6</v>
-      </c>
-      <c r="L56" t="n">
-        <v>6</v>
-      </c>
-      <c r="M56" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N56" t="n">
-        <v>1</v>
-      </c>
-      <c r="P56" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>1</v>
-      </c>
-      <c r="T56" t="n">
-        <v>1</v>
-      </c>
-      <c r="U56" t="n">
-        <v>1</v>
-      </c>
-      <c r="V56" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF56" t="n">
-        <v>5</v>
       </c>
       <c r="AG56" t="inlineStr">
         <is>
@@ -4357,7 +4414,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fotosíntesis</t>
+          <t>Flujo de energía y pirámides ecológicas</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4366,31 +4423,22 @@
         </is>
       </c>
       <c r="C57" t="n">
+        <v>5</v>
+      </c>
+      <c r="D57" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" t="n">
         <v>6</v>
       </c>
-      <c r="D57" t="n">
+      <c r="G57" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H57" t="n">
+        <v>5</v>
+      </c>
+      <c r="K57" t="n">
         <v>6</v>
-      </c>
-      <c r="E57" t="n">
-        <v>8</v>
-      </c>
-      <c r="F57" t="n">
-        <v>5</v>
-      </c>
-      <c r="G57" t="n">
-        <v>6</v>
-      </c>
-      <c r="H57" t="n">
-        <v>2</v>
-      </c>
-      <c r="I57" t="n">
-        <v>4</v>
-      </c>
-      <c r="J57" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K57" t="n">
-        <v>2</v>
       </c>
       <c r="L57" t="n">
         <v>6</v>
@@ -4401,21 +4449,12 @@
       <c r="N57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="n">
-        <v>1</v>
-      </c>
       <c r="P57" t="n">
         <v>1</v>
       </c>
       <c r="Q57" t="n">
         <v>1</v>
       </c>
-      <c r="R57" t="n">
-        <v>1</v>
-      </c>
-      <c r="S57" t="n">
-        <v>1</v>
-      </c>
       <c r="T57" t="n">
         <v>1</v>
       </c>
@@ -4426,7 +4465,7 @@
         <v>1</v>
       </c>
       <c r="AF57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AG57" t="inlineStr">
         <is>
@@ -4435,14 +4474,14 @@
       </c>
       <c r="AH57" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Genes y alelos</t>
+          <t>Fotosíntesis</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4456,20 +4495,35 @@
       <c r="D58" t="n">
         <v>6</v>
       </c>
+      <c r="E58" t="n">
+        <v>8</v>
+      </c>
       <c r="F58" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G58" t="n">
         <v>6</v>
       </c>
       <c r="H58" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I58" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J58" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
+      <c r="L58" t="n">
+        <v>6</v>
+      </c>
+      <c r="M58" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N58" t="n">
+        <v>1</v>
       </c>
       <c r="O58" t="n">
         <v>1</v>
@@ -4486,27 +4540,33 @@
       <c r="S58" t="n">
         <v>1</v>
       </c>
-      <c r="Z58" t="n">
+      <c r="T58" t="n">
+        <v>1</v>
+      </c>
+      <c r="U58" t="n">
+        <v>1</v>
+      </c>
+      <c r="V58" t="n">
         <v>1</v>
       </c>
       <c r="AF58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG58" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH58" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Genética humana y enfermedades hereditarias</t>
+          <t>Genes y alelos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4515,23 +4575,26 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D59" t="n">
+        <v>6</v>
       </c>
       <c r="F59" t="n">
         <v>8</v>
       </c>
       <c r="G59" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H59" t="n">
         <v>7</v>
       </c>
+      <c r="I59" t="n">
+        <v>8</v>
+      </c>
       <c r="J59" t="n">
         <v>7</v>
       </c>
-      <c r="M59" t="n">
-        <v>7</v>
-      </c>
       <c r="O59" t="n">
         <v>1</v>
       </c>
@@ -4541,21 +4604,21 @@
       <c r="Q59" t="n">
         <v>1</v>
       </c>
+      <c r="R59" t="n">
+        <v>1</v>
+      </c>
       <c r="S59" t="n">
         <v>1</v>
       </c>
-      <c r="V59" t="n">
-        <v>1</v>
-      </c>
       <c r="Z59" t="n">
         <v>1</v>
       </c>
       <c r="AF59" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH59" t="inlineStr">
@@ -4567,7 +4630,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Genotipo y fenotipo</t>
+          <t>Genética humana y enfermedades hereditarias</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4576,22 +4639,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>7</v>
-      </c>
-      <c r="D60" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>8</v>
       </c>
       <c r="G60" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H60" t="n">
-        <v>3</v>
-      </c>
-      <c r="I60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J60" t="n">
         <v>7</v>
@@ -4608,9 +4665,6 @@
       <c r="Q60" t="n">
         <v>1</v>
       </c>
-      <c r="R60" t="n">
-        <v>1</v>
-      </c>
       <c r="S60" t="n">
         <v>1</v>
       </c>
@@ -4621,7 +4675,7 @@
         <v>1</v>
       </c>
       <c r="AF60" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AG60" t="inlineStr">
         <is>
@@ -4637,7 +4691,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Grupos de alimentos y dieta balanceada</t>
+          <t>Genotipo y fenotipo</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4646,28 +4700,28 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
         <v>8</v>
       </c>
       <c r="G61" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H61" t="n">
-        <v>2</v>
-      </c>
-      <c r="K61" t="n">
-        <v>4</v>
-      </c>
-      <c r="L61" t="n">
-        <v>7.5</v>
+        <v>3</v>
+      </c>
+      <c r="I61" t="n">
+        <v>8</v>
+      </c>
+      <c r="J61" t="n">
+        <v>7</v>
       </c>
       <c r="M61" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="O61" t="n">
         <v>1</v>
@@ -4678,10 +4732,10 @@
       <c r="Q61" t="n">
         <v>1</v>
       </c>
-      <c r="T61" t="n">
-        <v>1</v>
-      </c>
-      <c r="U61" t="n">
+      <c r="R61" t="n">
+        <v>1</v>
+      </c>
+      <c r="S61" t="n">
         <v>1</v>
       </c>
       <c r="V61" t="n">
@@ -4691,11 +4745,11 @@
         <v>1</v>
       </c>
       <c r="AF61" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AG61" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH61" t="inlineStr">
@@ -4707,7 +4761,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Grupos de vertebrados</t>
+          <t>Grupos de alimentos y dieta balanceada</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4722,7 +4776,7 @@
         <v>2</v>
       </c>
       <c r="F62" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G62" t="n">
         <v>2</v>
@@ -4730,11 +4784,11 @@
       <c r="H62" t="n">
         <v>2</v>
       </c>
-      <c r="I62" t="n">
+      <c r="K62" t="n">
         <v>4</v>
       </c>
-      <c r="K62" t="n">
-        <v>2</v>
+      <c r="L62" t="n">
+        <v>7.5</v>
       </c>
       <c r="M62" t="n">
         <v>2.5</v>
@@ -4748,13 +4802,16 @@
       <c r="Q62" t="n">
         <v>1</v>
       </c>
-      <c r="R62" t="n">
-        <v>1</v>
-      </c>
       <c r="T62" t="n">
         <v>1</v>
       </c>
+      <c r="U62" t="n">
+        <v>1</v>
+      </c>
       <c r="V62" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z62" t="n">
         <v>1</v>
       </c>
       <c r="AF62" t="n">
@@ -4774,7 +4831,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Hábitat y ecosistemas comunes</t>
+          <t>Grupos de vertebrados</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4786,9 +4843,6 @@
         <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" t="n">
         <v>2</v>
       </c>
       <c r="F63" t="n">
@@ -4801,23 +4855,14 @@
         <v>2</v>
       </c>
       <c r="I63" t="n">
-        <v>2</v>
-      </c>
-      <c r="J63" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="K63" t="n">
         <v>2</v>
-      </c>
-      <c r="L63" t="n">
-        <v>6</v>
       </c>
       <c r="M63" t="n">
         <v>2.5</v>
       </c>
-      <c r="N63" t="n">
-        <v>1</v>
-      </c>
       <c r="O63" t="n">
         <v>1</v>
       </c>
@@ -4830,15 +4875,9 @@
       <c r="R63" t="n">
         <v>1</v>
       </c>
-      <c r="S63" t="n">
-        <v>1</v>
-      </c>
       <c r="T63" t="n">
         <v>1</v>
       </c>
-      <c r="U63" t="n">
-        <v>1</v>
-      </c>
       <c r="V63" t="n">
         <v>1</v>
       </c>
@@ -4847,7 +4886,7 @@
       </c>
       <c r="AG63" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH63" t="inlineStr">
@@ -4859,7 +4898,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Hábitos de vida saludable</t>
+          <t>Hábitat y ecosistemas comunes</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4871,6 +4910,9 @@
         <v>2</v>
       </c>
       <c r="D64" t="n">
+        <v>2</v>
+      </c>
+      <c r="E64" t="n">
         <v>2</v>
       </c>
       <c r="F64" t="n">
@@ -4882,14 +4924,23 @@
       <c r="H64" t="n">
         <v>2</v>
       </c>
+      <c r="I64" t="n">
+        <v>2</v>
+      </c>
       <c r="J64" t="n">
         <v>2.5</v>
       </c>
       <c r="K64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
-        <v>7.5</v>
+        <v>6</v>
+      </c>
+      <c r="M64" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N64" t="n">
+        <v>1</v>
       </c>
       <c r="O64" t="n">
         <v>1</v>
@@ -4900,6 +4951,9 @@
       <c r="Q64" t="n">
         <v>1</v>
       </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
       <c r="S64" t="n">
         <v>1</v>
       </c>
@@ -4909,7 +4963,7 @@
       <c r="U64" t="n">
         <v>1</v>
       </c>
-      <c r="Z64" t="n">
+      <c r="V64" t="n">
         <v>1</v>
       </c>
       <c r="AF64" t="n">
@@ -4929,7 +4983,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Herencia mendeliana</t>
+          <t>Hábitos de vida saludable</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4938,28 +4992,28 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G65" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H65" t="n">
-        <v>7</v>
-      </c>
-      <c r="I65" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>7</v>
-      </c>
-      <c r="M65" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="K65" t="n">
+        <v>4</v>
+      </c>
+      <c r="L65" t="n">
+        <v>7.5</v>
       </c>
       <c r="O65" t="n">
         <v>1</v>
@@ -4970,17 +5024,20 @@
       <c r="Q65" t="n">
         <v>1</v>
       </c>
-      <c r="R65" t="n">
-        <v>1</v>
-      </c>
       <c r="S65" t="n">
         <v>1</v>
       </c>
-      <c r="V65" t="n">
+      <c r="T65" t="n">
+        <v>1</v>
+      </c>
+      <c r="U65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z65" t="n">
         <v>1</v>
       </c>
       <c r="AF65" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG65" t="inlineStr">
         <is>
@@ -4996,7 +5053,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Herencia ligada al sexo, alelos múltiples y poligénica</t>
+          <t>Herencia de rasgos</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -5005,22 +5062,34 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="F66" t="n">
+        <v>8</v>
       </c>
       <c r="G66" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H66" t="n">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="I66" t="n">
+        <v>8</v>
       </c>
       <c r="J66" t="n">
         <v>7</v>
       </c>
+      <c r="L66" t="n">
+        <v>5</v>
+      </c>
       <c r="M66" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="O66" t="n">
+        <v>1</v>
       </c>
       <c r="P66" t="n">
         <v>1</v>
@@ -5028,13 +5097,16 @@
       <c r="Q66" t="n">
         <v>1</v>
       </c>
+      <c r="R66" t="n">
+        <v>1</v>
+      </c>
       <c r="S66" t="n">
         <v>1</v>
       </c>
+      <c r="U66" t="n">
+        <v>1</v>
+      </c>
       <c r="V66" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z66" t="n">
         <v>1</v>
       </c>
       <c r="AF66" t="n">
@@ -5047,14 +5119,14 @@
       </c>
       <c r="AH66" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Homeostasis</t>
+          <t>Herencia mendeliana</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5063,10 +5135,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
-      </c>
-      <c r="E67" t="n">
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="D67" t="n">
+        <v>7</v>
       </c>
       <c r="F67" t="n">
         <v>8</v>
@@ -5077,17 +5149,14 @@
       <c r="H67" t="n">
         <v>7</v>
       </c>
+      <c r="I67" t="n">
+        <v>8</v>
+      </c>
       <c r="J67" t="n">
         <v>7</v>
       </c>
-      <c r="K67" t="n">
-        <v>4</v>
-      </c>
       <c r="M67" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N67" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O67" t="n">
         <v>1</v>
@@ -5098,20 +5167,17 @@
       <c r="Q67" t="n">
         <v>1</v>
       </c>
+      <c r="R67" t="n">
+        <v>1</v>
+      </c>
       <c r="S67" t="n">
         <v>1</v>
       </c>
-      <c r="T67" t="n">
-        <v>1</v>
-      </c>
       <c r="V67" t="n">
         <v>1</v>
       </c>
-      <c r="Z67" t="n">
-        <v>1</v>
-      </c>
       <c r="AF67" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AG67" t="inlineStr">
         <is>
@@ -5127,7 +5193,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Impacto humano en los ecosistemas</t>
+          <t>Herencia ligada al sexo, alelos múltiples y poligénica</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -5136,37 +5202,22 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
-      </c>
-      <c r="F68" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="G68" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
-      </c>
-      <c r="I68" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J68" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K68" t="n">
-        <v>2</v>
-      </c>
-      <c r="L68" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="M68" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="O68" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="P68" t="n">
         <v>1</v>
@@ -5174,39 +5225,33 @@
       <c r="Q68" t="n">
         <v>1</v>
       </c>
-      <c r="R68" t="n">
-        <v>1</v>
-      </c>
       <c r="S68" t="n">
         <v>1</v>
       </c>
-      <c r="T68" t="n">
-        <v>1</v>
-      </c>
-      <c r="U68" t="n">
-        <v>1</v>
-      </c>
       <c r="V68" t="n">
         <v>1</v>
       </c>
+      <c r="Z68" t="n">
+        <v>1</v>
+      </c>
       <c r="AF68" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AG68" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH68" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>posterior</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Intercambio de gases en plantas</t>
+          <t>Homeostasis</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -5215,41 +5260,59 @@
         </is>
       </c>
       <c r="C69" t="n">
+        <v>9</v>
+      </c>
+      <c r="E69" t="n">
         <v>8</v>
       </c>
-      <c r="D69" t="n">
+      <c r="F69" t="n">
         <v>8</v>
       </c>
       <c r="G69" t="n">
-        <v>6</v>
-      </c>
-      <c r="I69" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H69" t="n">
         <v>7</v>
       </c>
       <c r="J69" t="n">
+        <v>7</v>
+      </c>
+      <c r="K69" t="n">
+        <v>4</v>
+      </c>
+      <c r="M69" t="n">
         <v>4.5</v>
       </c>
-      <c r="L69" t="n">
-        <v>5</v>
+      <c r="N69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O69" t="n">
+        <v>1</v>
       </c>
       <c r="P69" t="n">
         <v>1</v>
       </c>
-      <c r="R69" t="n">
+      <c r="Q69" t="n">
         <v>1</v>
       </c>
       <c r="S69" t="n">
         <v>1</v>
       </c>
-      <c r="U69" t="n">
+      <c r="T69" t="n">
+        <v>1</v>
+      </c>
+      <c r="V69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z69" t="n">
         <v>1</v>
       </c>
       <c r="AF69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG69" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH69" t="inlineStr">
@@ -5261,7 +5324,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Invertebrados e insectos</t>
+          <t>Impacto humano en los ecosistemas</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -5279,17 +5342,26 @@
         <v>2.5</v>
       </c>
       <c r="G70" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H70" t="n">
         <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="J70" t="n">
+        <v>2.5</v>
       </c>
       <c r="K70" t="n">
         <v>2</v>
       </c>
+      <c r="L70" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M70" t="n">
+        <v>2.5</v>
+      </c>
       <c r="O70" t="n">
         <v>1</v>
       </c>
@@ -5302,15 +5374,24 @@
       <c r="R70" t="n">
         <v>1</v>
       </c>
+      <c r="S70" t="n">
+        <v>1</v>
+      </c>
       <c r="T70" t="n">
         <v>1</v>
       </c>
+      <c r="U70" t="n">
+        <v>1</v>
+      </c>
+      <c r="V70" t="n">
+        <v>1</v>
+      </c>
       <c r="AF70" t="n">
         <v>2</v>
       </c>
       <c r="AG70" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH70" t="inlineStr">
@@ -5322,7 +5403,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>La célula como unidad de la vida</t>
+          <t>Intercambio de gases en plantas</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -5331,71 +5412,41 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D71" t="n">
-        <v>6</v>
-      </c>
-      <c r="E71" t="n">
-        <v>7</v>
-      </c>
-      <c r="F71" t="n">
         <v>8</v>
       </c>
       <c r="G71" t="n">
         <v>6</v>
       </c>
-      <c r="H71" t="n">
-        <v>5</v>
-      </c>
       <c r="I71" t="n">
         <v>7</v>
       </c>
       <c r="J71" t="n">
         <v>4.5</v>
       </c>
-      <c r="K71" t="n">
-        <v>7</v>
-      </c>
       <c r="L71" t="n">
         <v>5</v>
       </c>
-      <c r="M71" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N71" t="n">
-        <v>1</v>
-      </c>
-      <c r="O71" t="n">
-        <v>1</v>
-      </c>
       <c r="P71" t="n">
         <v>1</v>
       </c>
-      <c r="Q71" t="n">
-        <v>1</v>
-      </c>
       <c r="R71" t="n">
         <v>1</v>
       </c>
       <c r="S71" t="n">
         <v>1</v>
       </c>
-      <c r="T71" t="n">
-        <v>1</v>
-      </c>
       <c r="U71" t="n">
         <v>1</v>
       </c>
-      <c r="V71" t="n">
-        <v>1</v>
-      </c>
       <c r="AF71" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AG71" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH71" t="inlineStr">
@@ -5407,7 +5458,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Necesidades de los seres vivos</t>
+          <t>Invertebrados e insectos</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -5419,38 +5470,23 @@
         <v>2</v>
       </c>
       <c r="D72" t="n">
-        <v>2</v>
-      </c>
-      <c r="E72" t="n">
         <v>2</v>
       </c>
       <c r="F72" t="n">
         <v>2.5</v>
       </c>
       <c r="G72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H72" t="n">
         <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>4</v>
-      </c>
-      <c r="J72" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="K72" t="n">
         <v>2</v>
       </c>
-      <c r="L72" t="n">
-        <v>3</v>
-      </c>
-      <c r="M72" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N72" t="n">
-        <v>1</v>
-      </c>
       <c r="O72" t="n">
         <v>1</v>
       </c>
@@ -5463,16 +5499,7 @@
       <c r="R72" t="n">
         <v>1</v>
       </c>
-      <c r="S72" t="n">
-        <v>1</v>
-      </c>
       <c r="T72" t="n">
-        <v>1</v>
-      </c>
-      <c r="U72" t="n">
-        <v>1</v>
-      </c>
-      <c r="V72" t="n">
         <v>1</v>
       </c>
       <c r="AF72" t="n">
@@ -5492,7 +5519,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Niveles de organización de los seres vivos</t>
+          <t>La célula como unidad de la vida</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -5501,25 +5528,25 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D73" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E73" t="n">
         <v>7</v>
       </c>
       <c r="F73" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G73" t="n">
         <v>6</v>
       </c>
       <c r="H73" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I73" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J73" t="n">
         <v>4.5</v>
@@ -5528,7 +5555,7 @@
         <v>7</v>
       </c>
       <c r="L73" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="M73" t="n">
         <v>4.5</v>
@@ -5560,15 +5587,12 @@
       <c r="V73" t="n">
         <v>1</v>
       </c>
-      <c r="Z73" t="n">
-        <v>1</v>
-      </c>
       <c r="AF73" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH73" t="inlineStr">
@@ -5580,7 +5604,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Niveles de organización ecológica</t>
+          <t>Necesidades de los seres vivos</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -5589,31 +5613,40 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D74" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>2.5</v>
       </c>
       <c r="G74" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H74" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="I74" t="n">
+        <v>4</v>
       </c>
       <c r="J74" t="n">
         <v>2.5</v>
       </c>
       <c r="K74" t="n">
+        <v>2</v>
+      </c>
+      <c r="L74" t="n">
         <v>3</v>
       </c>
-      <c r="L74" t="n">
-        <v>6</v>
-      </c>
       <c r="M74" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="N74" t="n">
+        <v>1</v>
       </c>
       <c r="O74" t="n">
         <v>1</v>
@@ -5624,6 +5657,9 @@
       <c r="Q74" t="n">
         <v>1</v>
       </c>
+      <c r="R74" t="n">
+        <v>1</v>
+      </c>
       <c r="S74" t="n">
         <v>1</v>
       </c>
@@ -5637,11 +5673,11 @@
         <v>1</v>
       </c>
       <c r="AF74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG74" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH74" t="inlineStr">
@@ -5653,7 +5689,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Nutrición autótrofa y heterótrofa</t>
+          <t>Niveles de organización de los seres vivos</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -5662,34 +5698,40 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="E75" t="n">
+        <v>7</v>
       </c>
       <c r="F75" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="G75" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H75" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I75" t="n">
         <v>5</v>
       </c>
       <c r="J75" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L75" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="M75" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="N75" t="n">
+        <v>1</v>
       </c>
       <c r="O75" t="n">
         <v>1</v>
@@ -5715,8 +5757,11 @@
       <c r="V75" t="n">
         <v>1</v>
       </c>
+      <c r="Z75" t="n">
+        <v>1</v>
+      </c>
       <c r="AF75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AG75" t="inlineStr">
         <is>
@@ -5732,7 +5777,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Órganos de los sentidos</t>
+          <t>Niveles de organización ecológica</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -5747,25 +5792,25 @@
         <v>4</v>
       </c>
       <c r="F76" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G76" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H76" t="n">
-        <v>2</v>
-      </c>
-      <c r="I76" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J76" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="L76" t="n">
+        <v>6</v>
       </c>
       <c r="M76" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="O76" t="n">
         <v>1</v>
@@ -5776,13 +5821,13 @@
       <c r="Q76" t="n">
         <v>1</v>
       </c>
-      <c r="R76" t="n">
-        <v>1</v>
-      </c>
       <c r="S76" t="n">
         <v>1</v>
       </c>
       <c r="T76" t="n">
+        <v>1</v>
+      </c>
+      <c r="U76" t="n">
         <v>1</v>
       </c>
       <c r="V76" t="n">
@@ -5793,7 +5838,7 @@
       </c>
       <c r="AG76" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH76" t="inlineStr">
@@ -5805,7 +5850,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Partes de la planta y sus funciones</t>
+          <t>Nutrición autótrofa y heterótrofa</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5817,9 +5862,6 @@
         <v>2</v>
       </c>
       <c r="D77" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" t="n">
         <v>2</v>
       </c>
       <c r="F77" t="n">
@@ -5832,7 +5874,7 @@
         <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J77" t="n">
         <v>2.5</v>
@@ -5841,13 +5883,10 @@
         <v>2</v>
       </c>
       <c r="L77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M77" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N77" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O77" t="n">
         <v>1</v>
@@ -5874,11 +5913,11 @@
         <v>1</v>
       </c>
       <c r="AF77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG77" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH77" t="inlineStr">
@@ -5890,7 +5929,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Plantas y animales útiles al ser humano</t>
+          <t>Órganos de los sentidos</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -5899,22 +5938,25 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G78" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H78" t="n">
         <v>2</v>
       </c>
+      <c r="I78" t="n">
+        <v>7</v>
+      </c>
       <c r="J78" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="K78" t="n">
         <v>2</v>
@@ -5931,6 +5973,9 @@
       <c r="Q78" t="n">
         <v>1</v>
       </c>
+      <c r="R78" t="n">
+        <v>1</v>
+      </c>
       <c r="S78" t="n">
         <v>1</v>
       </c>
@@ -5941,11 +5986,11 @@
         <v>1</v>
       </c>
       <c r="AF78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH78" t="inlineStr">
@@ -5957,7 +6002,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Productores, consumidores y descomponedores</t>
+          <t>Partes de la planta y sus funciones</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5966,13 +6011,13 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>2.5</v>
@@ -5981,10 +6026,10 @@
         <v>2</v>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J79" t="n">
         <v>2.5</v>
@@ -5993,10 +6038,10 @@
         <v>2</v>
       </c>
       <c r="L79" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M79" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="N79" t="n">
         <v>1</v>
@@ -6026,7 +6071,7 @@
         <v>1</v>
       </c>
       <c r="AF79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG79" t="inlineStr">
         <is>
@@ -6042,7 +6087,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Reproducción humana y pubertad</t>
+          <t>Plantas y animales útiles al ser humano</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -6051,34 +6096,28 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D80" t="n">
-        <v>4</v>
-      </c>
-      <c r="E80" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G80" t="n">
-        <v>3</v>
+        <v>8.5</v>
       </c>
       <c r="H80" t="n">
-        <v>4</v>
-      </c>
-      <c r="I80" t="n">
-        <v>4</v>
-      </c>
-      <c r="L80" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="J80" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2</v>
       </c>
       <c r="M80" t="n">
-        <v>7</v>
-      </c>
-      <c r="N80" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="O80" t="n">
         <v>1</v>
@@ -6089,20 +6128,17 @@
       <c r="Q80" t="n">
         <v>1</v>
       </c>
-      <c r="R80" t="n">
-        <v>1</v>
-      </c>
-      <c r="U80" t="n">
+      <c r="S80" t="n">
+        <v>1</v>
+      </c>
+      <c r="T80" t="n">
         <v>1</v>
       </c>
       <c r="V80" t="n">
         <v>1</v>
       </c>
-      <c r="Z80" t="n">
-        <v>1</v>
-      </c>
       <c r="AF80" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG80" t="inlineStr">
         <is>
@@ -6118,7 +6154,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Reproducción sexual y asexual</t>
+          <t>Productores, consumidores y descomponedores</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -6127,31 +6163,37 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H81" t="n">
         <v>3</v>
       </c>
       <c r="I81" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="J81" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K81" t="n">
+        <v>2</v>
       </c>
       <c r="L81" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M81" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="N81" t="n">
         <v>1</v>
@@ -6168,17 +6210,20 @@
       <c r="R81" t="n">
         <v>1</v>
       </c>
+      <c r="S81" t="n">
+        <v>1</v>
+      </c>
+      <c r="T81" t="n">
+        <v>1</v>
+      </c>
       <c r="U81" t="n">
         <v>1</v>
       </c>
       <c r="V81" t="n">
         <v>1</v>
       </c>
-      <c r="Z81" t="n">
-        <v>1</v>
-      </c>
       <c r="AF81" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AG81" t="inlineStr">
         <is>
@@ -6194,7 +6239,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Requerimientos de materia y energía de la célula</t>
+          <t>Reproducción sexual de las plantas con flor</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6203,19 +6248,28 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D82" t="n">
+        <v>6</v>
+      </c>
+      <c r="E82" t="n">
+        <v>8</v>
+      </c>
+      <c r="F82" t="n">
+        <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H82" t="n">
-        <v>7</v>
-      </c>
-      <c r="J82" t="n">
-        <v>4.5</v>
+        <v>2</v>
+      </c>
+      <c r="I82" t="n">
+        <v>4</v>
       </c>
       <c r="K82" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L82" t="n">
         <v>5</v>
@@ -6223,13 +6277,19 @@
       <c r="M82" t="n">
         <v>7</v>
       </c>
+      <c r="N82" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" t="n">
+        <v>1</v>
+      </c>
       <c r="P82" t="n">
         <v>1</v>
       </c>
       <c r="Q82" t="n">
         <v>1</v>
       </c>
-      <c r="S82" t="n">
+      <c r="R82" t="n">
         <v>1</v>
       </c>
       <c r="T82" t="n">
@@ -6241,15 +6301,12 @@
       <c r="V82" t="n">
         <v>1</v>
       </c>
-      <c r="Z82" t="n">
-        <v>1</v>
-      </c>
       <c r="AF82" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG82" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH82" t="inlineStr">
@@ -6261,7 +6318,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Respiración celular</t>
+          <t>Reproducción humana y pubertad</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6270,35 +6327,29 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D83" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E83" t="n">
         <v>8</v>
       </c>
       <c r="F83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G83" t="n">
+        <v>3</v>
+      </c>
+      <c r="H83" t="n">
+        <v>4</v>
+      </c>
+      <c r="I83" t="n">
+        <v>4</v>
+      </c>
+      <c r="L83" t="n">
         <v>5</v>
       </c>
-      <c r="G83" t="n">
-        <v>6</v>
-      </c>
-      <c r="H83" t="n">
-        <v>7</v>
-      </c>
-      <c r="I83" t="n">
-        <v>7</v>
-      </c>
-      <c r="J83" t="n">
-        <v>7</v>
-      </c>
-      <c r="K83" t="n">
-        <v>7</v>
-      </c>
-      <c r="L83" t="n">
-        <v>6</v>
-      </c>
       <c r="M83" t="n">
         <v>7</v>
       </c>
@@ -6317,24 +6368,21 @@
       <c r="R83" t="n">
         <v>1</v>
       </c>
-      <c r="S83" t="n">
-        <v>1</v>
-      </c>
-      <c r="T83" t="n">
-        <v>1</v>
-      </c>
       <c r="U83" t="n">
         <v>1</v>
       </c>
       <c r="V83" t="n">
         <v>1</v>
       </c>
+      <c r="Z83" t="n">
+        <v>1</v>
+      </c>
       <c r="AF83" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AG83" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH83" t="inlineStr">
@@ -6346,7 +6394,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Respuesta de los seres vivos a estímulos</t>
+          <t>Reproducción sexual y asexual</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6355,10 +6403,10 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D84" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E84" t="n">
         <v>8</v>
@@ -6367,22 +6415,16 @@
         <v>8</v>
       </c>
       <c r="G84" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="H84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I84" t="n">
-        <v>3</v>
-      </c>
-      <c r="J84" t="n">
-        <v>7</v>
-      </c>
-      <c r="K84" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L84" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M84" t="n">
         <v>2.5</v>
@@ -6402,24 +6444,21 @@
       <c r="R84" t="n">
         <v>1</v>
       </c>
-      <c r="S84" t="n">
-        <v>1</v>
-      </c>
-      <c r="T84" t="n">
-        <v>1</v>
-      </c>
       <c r="U84" t="n">
         <v>1</v>
       </c>
       <c r="V84" t="n">
         <v>1</v>
       </c>
+      <c r="Z84" t="n">
+        <v>1</v>
+      </c>
       <c r="AF84" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH84" t="inlineStr">
@@ -6431,7 +6470,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Modelo estímulo-respuesta y retroalimentación negativa</t>
+          <t>Requerimientos de materia y energía de la célula</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6442,32 +6481,23 @@
       <c r="C85" t="n">
         <v>9</v>
       </c>
-      <c r="E85" t="n">
-        <v>8</v>
-      </c>
-      <c r="F85" t="n">
-        <v>8</v>
-      </c>
       <c r="G85" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H85" t="n">
         <v>7</v>
       </c>
-      <c r="I85" t="n">
-        <v>7</v>
-      </c>
       <c r="J85" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K85" t="n">
+        <v>7</v>
+      </c>
+      <c r="L85" t="n">
+        <v>5</v>
       </c>
       <c r="M85" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N85" t="n">
-        <v>1</v>
-      </c>
-      <c r="O85" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="P85" t="n">
         <v>1</v>
@@ -6475,33 +6505,39 @@
       <c r="Q85" t="n">
         <v>1</v>
       </c>
-      <c r="R85" t="n">
-        <v>1</v>
-      </c>
       <c r="S85" t="n">
         <v>1</v>
       </c>
+      <c r="T85" t="n">
+        <v>1</v>
+      </c>
+      <c r="U85" t="n">
+        <v>1</v>
+      </c>
       <c r="V85" t="n">
         <v>1</v>
       </c>
+      <c r="Z85" t="n">
+        <v>1</v>
+      </c>
       <c r="AF85" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH85" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Seres vivos y no vivos</t>
+          <t>Respiración celular</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -6510,31 +6546,37 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D86" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F86" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="G86" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H86" t="n">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="I86" t="n">
+        <v>7</v>
+      </c>
+      <c r="J86" t="n">
+        <v>7</v>
       </c>
       <c r="K86" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L86" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M86" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="N86" t="n">
         <v>1</v>
@@ -6548,6 +6590,12 @@
       <c r="Q86" t="n">
         <v>1</v>
       </c>
+      <c r="R86" t="n">
+        <v>1</v>
+      </c>
+      <c r="S86" t="n">
+        <v>1</v>
+      </c>
       <c r="T86" t="n">
         <v>1</v>
       </c>
@@ -6558,7 +6606,7 @@
         <v>1</v>
       </c>
       <c r="AF86" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AG86" t="inlineStr">
         <is>
@@ -6574,7 +6622,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Sistema circulatorio</t>
+          <t>Respuesta de los seres vivos a estímulos</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -6583,34 +6631,40 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D87" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="E87" t="n">
+        <v>8</v>
       </c>
       <c r="F87" t="n">
         <v>8</v>
       </c>
       <c r="G87" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="H87" t="n">
         <v>2</v>
       </c>
       <c r="I87" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J87" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="K87" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M87" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="N87" t="n">
+        <v>1</v>
       </c>
       <c r="O87" t="n">
         <v>1</v>
@@ -6636,15 +6690,12 @@
       <c r="V87" t="n">
         <v>1</v>
       </c>
-      <c r="Z87" t="n">
-        <v>1</v>
-      </c>
       <c r="AF87" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH87" t="inlineStr">
@@ -6656,7 +6707,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Sistema digestivo</t>
+          <t>Modelo estímulo-respuesta y retroalimentación negativa</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -6665,34 +6716,31 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>4</v>
-      </c>
-      <c r="D88" t="n">
-        <v>4</v>
+        <v>9</v>
+      </c>
+      <c r="E88" t="n">
+        <v>8</v>
       </c>
       <c r="F88" t="n">
         <v>8</v>
       </c>
       <c r="G88" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="H88" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I88" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J88" t="n">
+        <v>7</v>
+      </c>
+      <c r="M88" t="n">
         <v>4.5</v>
       </c>
-      <c r="K88" t="n">
-        <v>4</v>
-      </c>
-      <c r="L88" t="n">
-        <v>4</v>
-      </c>
-      <c r="M88" t="n">
-        <v>7</v>
+      <c r="N88" t="n">
+        <v>1</v>
       </c>
       <c r="O88" t="n">
         <v>1</v>
@@ -6709,20 +6757,11 @@
       <c r="S88" t="n">
         <v>1</v>
       </c>
-      <c r="T88" t="n">
-        <v>1</v>
-      </c>
-      <c r="U88" t="n">
-        <v>1</v>
-      </c>
       <c r="V88" t="n">
         <v>1</v>
       </c>
-      <c r="Z88" t="n">
-        <v>1</v>
-      </c>
       <c r="AF88" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AG88" t="inlineStr">
         <is>
@@ -6738,7 +6777,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sistema endocrino y hormonas</t>
+          <t>Seres vivos y no vivos</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -6747,25 +6786,31 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>9</v>
+        <v>2</v>
+      </c>
+      <c r="D89" t="n">
+        <v>2</v>
       </c>
       <c r="E89" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="G89" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J89" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="H89" t="n">
+        <v>2</v>
+      </c>
+      <c r="K89" t="n">
+        <v>2</v>
       </c>
       <c r="L89" t="n">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="M89" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="N89" t="n">
         <v>1</v>
@@ -6776,7 +6821,10 @@
       <c r="P89" t="n">
         <v>1</v>
       </c>
-      <c r="S89" t="n">
+      <c r="Q89" t="n">
+        <v>1</v>
+      </c>
+      <c r="T89" t="n">
         <v>1</v>
       </c>
       <c r="U89" t="n">
@@ -6785,11 +6833,8 @@
       <c r="V89" t="n">
         <v>1</v>
       </c>
-      <c r="Z89" t="n">
-        <v>1</v>
-      </c>
       <c r="AF89" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AG89" t="inlineStr">
         <is>
@@ -6805,7 +6850,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Sistema locomotor</t>
+          <t>Sistema circulatorio</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -6823,22 +6868,25 @@
         <v>8</v>
       </c>
       <c r="G90" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H90" t="n">
         <v>2</v>
       </c>
       <c r="I90" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J90" t="n">
         <v>4.5</v>
       </c>
       <c r="K90" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="L90" t="n">
+        <v>4</v>
       </c>
       <c r="M90" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="O90" t="n">
         <v>1</v>
@@ -6858,7 +6906,13 @@
       <c r="T90" t="n">
         <v>1</v>
       </c>
+      <c r="U90" t="n">
+        <v>1</v>
+      </c>
       <c r="V90" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z90" t="n">
         <v>1</v>
       </c>
       <c r="AF90" t="n">
@@ -6878,7 +6932,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Sistema respiratorio</t>
+          <t>Sistema digestivo</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -6887,19 +6941,19 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H91" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I91" t="n">
         <v>5</v>
@@ -6948,7 +7002,7 @@
       </c>
       <c r="AG91" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH91" t="inlineStr">
@@ -6960,7 +7014,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Tejidos animales</t>
+          <t>Sistema endocrino y hormonas</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -6969,13 +7023,10 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>6</v>
-      </c>
-      <c r="D92" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F92" t="n">
         <v>8</v>
@@ -6983,7 +7034,13 @@
       <c r="G92" t="n">
         <v>8.5</v>
       </c>
-      <c r="H92" t="n">
+      <c r="J92" t="n">
+        <v>7</v>
+      </c>
+      <c r="L92" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M92" t="n">
         <v>7</v>
       </c>
       <c r="N92" t="n">
@@ -6995,30 +7052,36 @@
       <c r="P92" t="n">
         <v>1</v>
       </c>
-      <c r="Q92" t="n">
+      <c r="S92" t="n">
+        <v>1</v>
+      </c>
+      <c r="U92" t="n">
+        <v>1</v>
+      </c>
+      <c r="V92" t="n">
         <v>1</v>
       </c>
       <c r="Z92" t="n">
         <v>1</v>
       </c>
       <c r="AF92" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="AG92" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH92" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Tejidos vegetales</t>
+          <t>Sistema locomotor</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -7027,34 +7090,31 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D93" t="n">
-        <v>8</v>
-      </c>
-      <c r="E93" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>8</v>
       </c>
       <c r="G93" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="H93" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="I93" t="n">
+        <v>3</v>
       </c>
       <c r="J93" t="n">
         <v>4.5</v>
       </c>
-      <c r="L93" t="n">
-        <v>7.5</v>
+      <c r="K93" t="n">
+        <v>2</v>
       </c>
       <c r="M93" t="n">
-        <v>7</v>
-      </c>
-      <c r="N93" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="O93" t="n">
         <v>1</v>
@@ -7065,17 +7125,20 @@
       <c r="Q93" t="n">
         <v>1</v>
       </c>
+      <c r="R93" t="n">
+        <v>1</v>
+      </c>
       <c r="S93" t="n">
         <v>1</v>
       </c>
-      <c r="U93" t="n">
+      <c r="T93" t="n">
         <v>1</v>
       </c>
       <c r="V93" t="n">
         <v>1</v>
       </c>
       <c r="AF93" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AG93" t="inlineStr">
         <is>
@@ -7091,7 +7154,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Transporte en plantas: xilema y floema</t>
+          <t>Sistema respiratorio</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -7100,16 +7163,19 @@
         </is>
       </c>
       <c r="C94" t="n">
+        <v>3</v>
+      </c>
+      <c r="D94" t="n">
+        <v>3</v>
+      </c>
+      <c r="F94" t="n">
+        <v>8</v>
+      </c>
+      <c r="G94" t="n">
         <v>6</v>
       </c>
-      <c r="D94" t="n">
-        <v>6</v>
-      </c>
-      <c r="G94" t="n">
-        <v>2</v>
-      </c>
       <c r="H94" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I94" t="n">
         <v>5</v>
@@ -7117,12 +7183,18 @@
       <c r="J94" t="n">
         <v>4.5</v>
       </c>
+      <c r="K94" t="n">
+        <v>4</v>
+      </c>
       <c r="L94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M94" t="n">
         <v>7</v>
       </c>
+      <c r="O94" t="n">
+        <v>1</v>
+      </c>
       <c r="P94" t="n">
         <v>1</v>
       </c>
@@ -7135,18 +7207,24 @@
       <c r="S94" t="n">
         <v>1</v>
       </c>
+      <c r="T94" t="n">
+        <v>1</v>
+      </c>
       <c r="U94" t="n">
         <v>1</v>
       </c>
       <c r="V94" t="n">
         <v>1</v>
       </c>
+      <c r="Z94" t="n">
+        <v>1</v>
+      </c>
       <c r="AF94" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AG94" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH94" t="inlineStr">
@@ -7158,7 +7236,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Variación genética en la descendencia</t>
+          <t>Tejidos animales</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -7172,26 +7250,20 @@
       <c r="D95" t="n">
         <v>6</v>
       </c>
+      <c r="E95" t="n">
+        <v>7</v>
+      </c>
       <c r="F95" t="n">
         <v>8</v>
       </c>
       <c r="G95" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="H95" t="n">
         <v>7</v>
       </c>
-      <c r="I95" t="n">
-        <v>8</v>
-      </c>
-      <c r="K95" t="n">
-        <v>5</v>
-      </c>
-      <c r="L95" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="M95" t="n">
-        <v>4.5</v>
+      <c r="N95" t="n">
+        <v>1</v>
       </c>
       <c r="O95" t="n">
         <v>1</v>
@@ -7202,48 +7274,39 @@
       <c r="Q95" t="n">
         <v>1</v>
       </c>
-      <c r="R95" t="n">
-        <v>1</v>
-      </c>
-      <c r="T95" t="n">
-        <v>1</v>
-      </c>
-      <c r="U95" t="n">
-        <v>1</v>
-      </c>
-      <c r="V95" t="n">
+      <c r="Z95" t="n">
         <v>1</v>
       </c>
       <c r="AF95" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AG95" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH95" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Célula animal y célula vegetal</t>
+          <t>Tejidos vegetales</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D96" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E96" t="n">
         <v>7</v>
@@ -7252,20 +7315,14 @@
         <v>8</v>
       </c>
       <c r="G96" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="H96" t="n">
-        <v>5</v>
-      </c>
-      <c r="I96" t="n">
         <v>7</v>
       </c>
       <c r="J96" t="n">
         <v>4.5</v>
       </c>
-      <c r="K96" t="n">
-        <v>7</v>
-      </c>
       <c r="L96" t="n">
         <v>7.5</v>
       </c>
@@ -7284,15 +7341,9 @@
       <c r="Q96" t="n">
         <v>1</v>
       </c>
-      <c r="R96" t="n">
-        <v>1</v>
-      </c>
       <c r="S96" t="n">
         <v>1</v>
       </c>
-      <c r="T96" t="n">
-        <v>1</v>
-      </c>
       <c r="U96" t="n">
         <v>1</v>
       </c>
@@ -7300,7 +7351,7 @@
         <v>1</v>
       </c>
       <c r="AF96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AG96" t="inlineStr">
         <is>
@@ -7309,62 +7360,86 @@
       </c>
       <c r="AH96" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Especiación y macroevolución</t>
+          <t>Transporte en plantas: xilema y floema</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C97" t="n">
+        <v>6</v>
+      </c>
+      <c r="D97" t="n">
+        <v>6</v>
+      </c>
+      <c r="G97" t="n">
+        <v>2</v>
+      </c>
+      <c r="H97" t="n">
+        <v>7</v>
+      </c>
+      <c r="I97" t="n">
         <v>5</v>
       </c>
-      <c r="D97" t="n">
+      <c r="J97" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L97" t="n">
         <v>5</v>
       </c>
-      <c r="F97" t="n">
+      <c r="M97" t="n">
+        <v>7</v>
+      </c>
+      <c r="P97" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>1</v>
+      </c>
+      <c r="R97" t="n">
+        <v>1</v>
+      </c>
+      <c r="S97" t="n">
+        <v>1</v>
+      </c>
+      <c r="U97" t="n">
+        <v>1</v>
+      </c>
+      <c r="V97" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF97" t="n">
         <v>8</v>
       </c>
-      <c r="G97" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="O97" t="n">
-        <v>1</v>
-      </c>
-      <c r="P97" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF97" t="n">
-        <v>11</v>
-      </c>
       <c r="AG97" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH97" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Estructuras celulares básicas</t>
+          <t>Variación genética en la descendencia</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -7373,35 +7448,26 @@
       <c r="D98" t="n">
         <v>6</v>
       </c>
-      <c r="E98" t="n">
-        <v>7</v>
-      </c>
       <c r="F98" t="n">
         <v>8</v>
       </c>
       <c r="G98" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H98" t="n">
+        <v>7</v>
+      </c>
+      <c r="I98" t="n">
+        <v>8</v>
+      </c>
+      <c r="K98" t="n">
         <v>5</v>
-      </c>
-      <c r="I98" t="n">
-        <v>7</v>
-      </c>
-      <c r="J98" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K98" t="n">
-        <v>7</v>
       </c>
       <c r="L98" t="n">
         <v>7.5</v>
       </c>
       <c r="M98" t="n">
-        <v>7</v>
-      </c>
-      <c r="N98" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="O98" t="n">
         <v>1</v>
@@ -7415,9 +7481,6 @@
       <c r="R98" t="n">
         <v>1</v>
       </c>
-      <c r="S98" t="n">
-        <v>1</v>
-      </c>
       <c r="T98" t="n">
         <v>1</v>
       </c>
@@ -7427,11 +7490,8 @@
       <c r="V98" t="n">
         <v>1</v>
       </c>
-      <c r="Z98" t="n">
-        <v>1</v>
-      </c>
       <c r="AF98" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AG98" t="inlineStr">
         <is>
@@ -7440,121 +7500,85 @@
       </c>
       <c r="AH98" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Herencia de rasgos</t>
+          <t>Especies clave</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>no_aplica</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D99" t="n">
-        <v>6</v>
-      </c>
-      <c r="F99" t="n">
-        <v>8</v>
-      </c>
-      <c r="G99" t="n">
-        <v>2</v>
-      </c>
-      <c r="H99" t="n">
+        <v>7</v>
+      </c>
+      <c r="K99" t="n">
         <v>3</v>
       </c>
-      <c r="I99" t="n">
-        <v>8</v>
-      </c>
-      <c r="J99" t="n">
-        <v>7</v>
-      </c>
-      <c r="L99" t="n">
-        <v>5</v>
-      </c>
-      <c r="M99" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="O99" t="n">
-        <v>1</v>
-      </c>
-      <c r="P99" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q99" t="n">
-        <v>1</v>
-      </c>
-      <c r="R99" t="n">
-        <v>1</v>
-      </c>
-      <c r="S99" t="n">
-        <v>1</v>
-      </c>
-      <c r="U99" t="n">
-        <v>1</v>
-      </c>
-      <c r="V99" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF99" t="n">
-        <v>10</v>
+      <c r="T99" t="n">
+        <v>1</v>
       </c>
       <c r="AG99" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH99" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>no_aplica</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Mutaciones</t>
+          <t>Adaptaciones fisiológicas</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D100" t="n">
-        <v>7</v>
-      </c>
-      <c r="G100" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="M100" t="n">
-        <v>7</v>
-      </c>
-      <c r="P100" t="n">
-        <v>1</v>
-      </c>
-      <c r="V100" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z100" t="n">
+        <v>8</v>
+      </c>
+      <c r="F100" t="n">
+        <v>8</v>
+      </c>
+      <c r="H100" t="n">
+        <v>3</v>
+      </c>
+      <c r="K100" t="n">
+        <v>2</v>
+      </c>
+      <c r="O100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>1</v>
+      </c>
+      <c r="T100" t="n">
         <v>1</v>
       </c>
       <c r="AF100" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AG100" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH100" t="inlineStr">
@@ -7566,12 +7590,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Reproducción sexual de las plantas con flor</t>
+          <t>Biotecnología vegetal y agroindustria</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>incierto</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -7580,84 +7604,51 @@
       <c r="D101" t="n">
         <v>6</v>
       </c>
-      <c r="E101" t="n">
-        <v>8</v>
-      </c>
       <c r="F101" t="n">
         <v>8</v>
       </c>
       <c r="G101" t="n">
-        <v>2</v>
-      </c>
-      <c r="H101" t="n">
-        <v>2</v>
-      </c>
-      <c r="I101" t="n">
-        <v>4</v>
-      </c>
-      <c r="K101" t="n">
-        <v>2</v>
-      </c>
-      <c r="L101" t="n">
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="M101" t="n">
         <v>7</v>
       </c>
-      <c r="N101" t="n">
-        <v>1</v>
-      </c>
       <c r="O101" t="n">
         <v>1</v>
       </c>
       <c r="P101" t="n">
         <v>1</v>
       </c>
-      <c r="Q101" t="n">
-        <v>1</v>
-      </c>
-      <c r="R101" t="n">
-        <v>1</v>
-      </c>
-      <c r="T101" t="n">
-        <v>1</v>
-      </c>
-      <c r="U101" t="n">
-        <v>1</v>
-      </c>
       <c r="V101" t="n">
         <v>1</v>
       </c>
       <c r="AF101" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="AG101" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH101" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Especies clave</t>
+          <t>Capacidad de carga</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>no_aplica</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>7</v>
-      </c>
-      <c r="D102" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K102" t="n">
         <v>3</v>
@@ -7665,21 +7656,24 @@
       <c r="T102" t="n">
         <v>1</v>
       </c>
+      <c r="AF102" t="n">
+        <v>11</v>
+      </c>
       <c r="AG102" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH102" t="inlineStr">
         <is>
-          <t>no_aplica</t>
+          <t>posterior</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Adaptaciones fisiológicas</t>
+          <t>Ciclo del nitrógeno</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -7688,35 +7682,32 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>8</v>
-      </c>
-      <c r="D103" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F103" t="n">
         <v>8</v>
       </c>
-      <c r="H103" t="n">
-        <v>3</v>
+      <c r="G103" t="n">
+        <v>8.5</v>
       </c>
       <c r="K103" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O103" t="n">
         <v>1</v>
       </c>
-      <c r="Q103" t="n">
+      <c r="P103" t="n">
         <v>1</v>
       </c>
       <c r="T103" t="n">
         <v>1</v>
       </c>
       <c r="AF103" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG103" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH103" t="inlineStr">
@@ -7728,7 +7719,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Capacidad de carga</t>
+          <t>Propagación de enfermedades y control de brotes</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -7737,16 +7728,37 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>11</v>
-      </c>
-      <c r="K104" t="n">
+        <v>9</v>
+      </c>
+      <c r="G104" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H104" t="n">
         <v>3</v>
       </c>
-      <c r="T104" t="n">
+      <c r="J104" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L104" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>1</v>
+      </c>
+      <c r="S104" t="n">
+        <v>1</v>
+      </c>
+      <c r="U104" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z104" t="n">
         <v>1</v>
       </c>
       <c r="AF104" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG104" t="inlineStr">
         <is>
@@ -7762,7 +7774,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Ciclo del nitrógeno</t>
+          <t>Especiación y macroevolución</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -7771,7 +7783,10 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="D105" t="n">
+        <v>5</v>
       </c>
       <c r="F105" t="n">
         <v>8</v>
@@ -7779,24 +7794,18 @@
       <c r="G105" t="n">
         <v>8.5</v>
       </c>
-      <c r="K105" t="n">
-        <v>6</v>
-      </c>
       <c r="O105" t="n">
         <v>1</v>
       </c>
       <c r="P105" t="n">
         <v>1</v>
       </c>
-      <c r="T105" t="n">
-        <v>1</v>
-      </c>
       <c r="AF105" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AG105" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH105" t="inlineStr">
@@ -7808,7 +7817,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Propagación de enfermedades y control de brotes</t>
+          <t>Eutrofización</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -7817,41 +7826,17 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
-      </c>
-      <c r="G106" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H106" t="n">
-        <v>3</v>
-      </c>
-      <c r="J106" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L106" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="P106" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q106" t="n">
-        <v>1</v>
-      </c>
-      <c r="S106" t="n">
-        <v>1</v>
-      </c>
-      <c r="U106" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z106" t="n">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="D106" t="n">
+        <v>7</v>
       </c>
       <c r="AF106" t="n">
         <v>9</v>
       </c>
       <c r="AG106" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH106" t="inlineStr">
@@ -7863,7 +7848,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Eutrofización</t>
+          <t>Evidencias de la evolución</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -7872,17 +7857,38 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>7</v>
-      </c>
-      <c r="D107" t="n">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="F107" t="n">
+        <v>8</v>
+      </c>
+      <c r="G107" t="n">
+        <v>4</v>
+      </c>
+      <c r="I107" t="n">
+        <v>8</v>
+      </c>
+      <c r="M107" t="n">
+        <v>7</v>
+      </c>
+      <c r="O107" t="n">
+        <v>1</v>
+      </c>
+      <c r="P107" t="n">
+        <v>1</v>
+      </c>
+      <c r="R107" t="n">
+        <v>1</v>
+      </c>
+      <c r="V107" t="n">
+        <v>1</v>
       </c>
       <c r="AF107" t="n">
         <v>9</v>
       </c>
       <c r="AG107" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH107" t="inlineStr">
@@ -7894,7 +7900,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Evidencias de la evolución</t>
+          <t>Fases de la fotosíntesis y ciclo de Calvin</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -7903,38 +7909,23 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D108" t="n">
+        <v>6</v>
       </c>
       <c r="F108" t="n">
         <v>8</v>
       </c>
-      <c r="G108" t="n">
-        <v>4</v>
-      </c>
-      <c r="I108" t="n">
-        <v>8</v>
-      </c>
-      <c r="M108" t="n">
-        <v>7</v>
-      </c>
       <c r="O108" t="n">
         <v>1</v>
       </c>
-      <c r="P108" t="n">
-        <v>1</v>
-      </c>
-      <c r="R108" t="n">
-        <v>1</v>
-      </c>
-      <c r="V108" t="n">
-        <v>1</v>
-      </c>
       <c r="AF108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG108" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH108" t="inlineStr">
@@ -7946,7 +7937,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Fases de la fotosíntesis y ciclo de Calvin</t>
+          <t>Secuenciación del ADN y perfiles genéticos</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -7955,15 +7946,18 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>6</v>
-      </c>
-      <c r="D109" t="n">
-        <v>6</v>
-      </c>
-      <c r="F109" t="n">
-        <v>8</v>
-      </c>
-      <c r="O109" t="n">
+        <v>9</v>
+      </c>
+      <c r="G109" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H109" t="n">
+        <v>7</v>
+      </c>
+      <c r="P109" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q109" t="n">
         <v>1</v>
       </c>
       <c r="AF109" t="n">
@@ -7971,7 +7965,7 @@
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
       <c r="AH109" t="inlineStr">
@@ -7983,7 +7977,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Secuenciación del ADN y perfiles genéticos</t>
+          <t>Impulso nervioso y sinapsis</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -7992,18 +7986,18 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
-      </c>
-      <c r="G110" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H110" t="n">
-        <v>7</v>
-      </c>
-      <c r="P110" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q110" t="n">
+        <v>10</v>
+      </c>
+      <c r="F110" t="n">
+        <v>8</v>
+      </c>
+      <c r="J110" t="n">
+        <v>7</v>
+      </c>
+      <c r="O110" t="n">
+        <v>1</v>
+      </c>
+      <c r="S110" t="n">
         <v>1</v>
       </c>
       <c r="AF110" t="n">
@@ -8023,7 +8017,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Impulso nervioso y sinapsis</t>
+          <t>Ingeniería genética y ADN recombinante</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -8032,22 +8026,37 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F111" t="n">
         <v>8</v>
       </c>
-      <c r="J111" t="n">
+      <c r="G111" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H111" t="n">
+        <v>7</v>
+      </c>
+      <c r="M111" t="n">
         <v>7</v>
       </c>
       <c r="O111" t="n">
         <v>1</v>
       </c>
-      <c r="S111" t="n">
+      <c r="P111" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>1</v>
+      </c>
+      <c r="V111" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z111" t="n">
         <v>1</v>
       </c>
       <c r="AF111" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AG111" t="inlineStr">
         <is>
@@ -8063,7 +8072,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Ingeniería genética y ADN recombinante</t>
+          <t>Inmunidad adaptativa</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -8072,29 +8081,17 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>11</v>
-      </c>
-      <c r="F112" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G112" t="n">
         <v>8.5</v>
       </c>
-      <c r="H112" t="n">
-        <v>7</v>
-      </c>
       <c r="M112" t="n">
         <v>7</v>
       </c>
-      <c r="O112" t="n">
-        <v>1</v>
-      </c>
       <c r="P112" t="n">
         <v>1</v>
       </c>
-      <c r="Q112" t="n">
-        <v>1</v>
-      </c>
       <c r="V112" t="n">
         <v>1</v>
       </c>
@@ -8102,7 +8099,7 @@
         <v>1</v>
       </c>
       <c r="AF112" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AG112" t="inlineStr">
         <is>
@@ -8118,7 +8115,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Inmunidad adaptativa</t>
+          <t>Inmunidad innata</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -8141,9 +8138,6 @@
       <c r="V113" t="n">
         <v>1</v>
       </c>
-      <c r="Z113" t="n">
-        <v>1</v>
-      </c>
       <c r="AF113" t="n">
         <v>10</v>
       </c>
@@ -8161,7 +8155,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Inmunidad innata</t>
+          <t>Mutaciones</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -8170,7 +8164,10 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="D114" t="n">
+        <v>7</v>
       </c>
       <c r="G114" t="n">
         <v>8.5</v>
@@ -8184,12 +8181,15 @@
       <c r="V114" t="n">
         <v>1</v>
       </c>
+      <c r="Z114" t="n">
+        <v>1</v>
+      </c>
       <c r="AF114" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AG114" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH114" t="inlineStr">

</xml_diff>